<commit_message>
- Errores arreglados del doc 2 (05-05-2024)
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -647,7 +647,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1465" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1465" uniqueCount="330">
   <si>
     <t xml:space="preserve">Activo</t>
   </si>
@@ -1426,7 +1426,7 @@
     <t xml:space="preserve">LA293 SCL PUQ</t>
   </si>
   <si>
-    <t xml:space="preserve">23:50 03:14+1</t>
+    <t xml:space="preserve">23:50 03:14+2</t>
   </si>
   <si>
     <t xml:space="preserve">DAP PUQ WPU</t>
@@ -1448,6 +1448,9 @@
   </si>
   <si>
     <t xml:space="preserve">Qantas Airways</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23:50 03:14+1</t>
   </si>
   <si>
     <t xml:space="preserve"> CHRISTOPHER JOHN</t>
@@ -5918,7 +5921,7 @@
         <v>45668</v>
       </c>
       <c r="AM13" s="46" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="AN13" s="47" t="s">
         <v>260</v>
@@ -6097,20 +6100,20 @@
         <v>113</v>
       </c>
       <c r="K14" s="41" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="L14" s="41" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="M14" s="39"/>
       <c r="N14" s="41" t="s">
         <v>145</v>
       </c>
       <c r="O14" s="41" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="P14" s="40" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="Q14" s="43" t="n">
         <v>32894</v>
@@ -6169,13 +6172,13 @@
         <v>0.590277777777778</v>
       </c>
       <c r="AK14" s="45" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="AL14" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM14" s="46" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="AN14" s="47" t="s">
         <v>260</v>
@@ -6354,20 +6357,20 @@
         <v>113</v>
       </c>
       <c r="K15" s="41" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="L15" s="41" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="M15" s="39"/>
       <c r="N15" s="41" t="s">
         <v>145</v>
       </c>
       <c r="O15" s="41" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="P15" s="40" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="Q15" s="43" t="n">
         <v>32113</v>
@@ -6426,13 +6429,13 @@
         <v>0.590277777777778</v>
       </c>
       <c r="AK15" s="45" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="AL15" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM15" s="46" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="AN15" s="47" t="s">
         <v>260</v>
@@ -6611,20 +6614,20 @@
         <v>113</v>
       </c>
       <c r="K16" s="41" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="L16" s="41" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="M16" s="39"/>
       <c r="N16" s="41" t="s">
         <v>145</v>
       </c>
       <c r="O16" s="41" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="P16" s="40" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="Q16" s="43" t="n">
         <v>35754</v>
@@ -6689,7 +6692,7 @@
         <v>45668</v>
       </c>
       <c r="AM16" s="46" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="AN16" s="47" t="s">
         <v>260</v>
@@ -6734,7 +6737,7 @@
         <v>151</v>
       </c>
       <c r="BB16" s="40" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="BC16" s="40" t="s">
         <v>176</v>
@@ -6758,7 +6761,7 @@
       <c r="BJ16" s="43"/>
       <c r="BK16" s="40"/>
       <c r="BL16" s="40" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="BM16" s="40" t="s">
         <v>135</v>
@@ -6868,10 +6871,10 @@
         <v>113</v>
       </c>
       <c r="K17" s="41" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="L17" s="41" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="M17" s="39"/>
       <c r="N17" s="41" t="s">
@@ -6881,7 +6884,7 @@
         <v>201</v>
       </c>
       <c r="P17" s="40" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="Q17" s="43" t="n">
         <v>33264</v>
@@ -6895,22 +6898,22 @@
       <c r="T17" s="41"/>
       <c r="U17" s="40"/>
       <c r="V17" s="41" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="W17" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X17" s="42" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="Y17" s="40" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="Z17" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA17" s="42" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="AB17" s="40" t="s">
         <v>147</v>
@@ -6940,13 +6943,13 @@
         <v>0.590277777777778</v>
       </c>
       <c r="AK17" s="45" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="AL17" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM17" s="46" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="AN17" s="47" t="s">
         <v>260</v>
@@ -7125,20 +7128,20 @@
         <v>113</v>
       </c>
       <c r="K18" s="41" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="L18" s="41" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="M18" s="39"/>
       <c r="N18" s="41" t="s">
         <v>145</v>
       </c>
       <c r="O18" s="41" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="P18" s="40" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="Q18" s="43" t="n">
         <v>28156</v>
@@ -7152,13 +7155,13 @@
       <c r="T18" s="41"/>
       <c r="U18" s="40"/>
       <c r="V18" s="41" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="W18" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X18" s="42" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="Y18" s="40" t="s">
         <v>216</v>
@@ -7203,7 +7206,7 @@
         <v>45668</v>
       </c>
       <c r="AM18" s="46" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="AN18" s="47" t="s">
         <v>260</v>
@@ -7248,7 +7251,7 @@
         <v>151</v>
       </c>
       <c r="BB18" s="40" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="BC18" s="40" t="s">
         <v>176</v>
@@ -7272,7 +7275,7 @@
       <c r="BJ18" s="43"/>
       <c r="BK18" s="40"/>
       <c r="BL18" s="40" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="BM18" s="40" t="s">
         <v>135</v>
@@ -7382,19 +7385,19 @@
         <v>113</v>
       </c>
       <c r="K19" s="58" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L19" s="58" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="N19" s="58" t="s">
         <v>145</v>
       </c>
       <c r="O19" s="58" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="P19" s="48" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="Q19" s="43" t="n">
         <v>33314</v>
@@ -7408,13 +7411,13 @@
       <c r="T19" s="58"/>
       <c r="U19" s="48"/>
       <c r="V19" s="58" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="W19" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="X19" s="59" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="Y19" s="48" t="s">
         <v>216</v>
@@ -7459,7 +7462,7 @@
         <v>45668</v>
       </c>
       <c r="AM19" s="62" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="AN19" s="47" t="s">
         <v>260</v>
@@ -7504,7 +7507,7 @@
         <v>151</v>
       </c>
       <c r="BB19" s="48" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="BC19" s="40" t="s">
         <v>176</v>
@@ -7528,7 +7531,7 @@
       <c r="BJ19" s="60"/>
       <c r="BK19" s="48"/>
       <c r="BL19" s="48" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="BM19" s="40" t="s">
         <v>135</v>
@@ -7635,19 +7638,19 @@
         <v>113</v>
       </c>
       <c r="K20" s="58" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L20" s="58" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="N20" s="58" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="O20" s="58" t="s">
         <v>162</v>
       </c>
       <c r="P20" s="48" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="Q20" s="43" t="n">
         <v>33003</v>
@@ -7659,31 +7662,31 @@
       <c r="T20" s="58"/>
       <c r="U20" s="48"/>
       <c r="V20" s="58" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="W20" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="X20" s="59" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="Y20" s="48" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="Z20" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="AA20" s="59" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="AB20" s="48" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="AC20" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="AD20" s="59" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="AE20" s="48" t="s">
         <v>147</v>
@@ -7695,7 +7698,7 @@
         <v>147</v>
       </c>
       <c r="AH20" s="58" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="AI20" s="59" t="n">
         <v>45668</v>
@@ -7704,13 +7707,13 @@
         <v>0.225694444444444</v>
       </c>
       <c r="AK20" s="61" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="AL20" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM20" s="62" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="AN20" s="47" t="s">
         <v>260</v>
@@ -7886,19 +7889,19 @@
         <v>113</v>
       </c>
       <c r="K21" s="58" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="L21" s="58" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="N21" s="58" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="O21" s="58" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="P21" s="48" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="Q21" s="43" t="n">
         <v>32465</v>
@@ -7912,31 +7915,31 @@
       <c r="T21" s="58"/>
       <c r="U21" s="48"/>
       <c r="V21" s="58" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="W21" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="X21" s="59" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="Y21" s="48" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="Z21" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="AA21" s="59" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="AB21" s="48" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="AC21" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="AD21" s="59" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="AE21" s="48" t="s">
         <v>147</v>
@@ -7963,7 +7966,7 @@
         <v>45668</v>
       </c>
       <c r="AM21" s="62" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="AN21" s="47" t="s">
         <v>260</v>
@@ -8008,7 +8011,7 @@
         <v>151</v>
       </c>
       <c r="BB21" s="48" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="BC21" s="40" t="s">
         <v>176</v>
@@ -8032,7 +8035,7 @@
       <c r="BJ21" s="60"/>
       <c r="BK21" s="48"/>
       <c r="BL21" s="48" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="BM21" s="40" t="s">
         <v>135</v>
@@ -29148,10 +29151,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D1" s="99" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E1" s="99" t="s">
         <v>4</v>
@@ -29160,13 +29163,13 @@
         <v>5</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="H1" s="11" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="15" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="J1" s="15" t="s">
         <v>9</v>
@@ -29181,7 +29184,7 @@
         <v>12</v>
       </c>
       <c r="N1" s="32" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="O1" s="32" t="s">
         <v>14</v>
@@ -29465,7 +29468,7 @@
         <v>115</v>
       </c>
       <c r="M2" s="32" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="N2" s="32" t="s">
         <v>117</v>
@@ -29744,25 +29747,25 @@
         <v>113</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="O3" s="2" t="s">
         <v>162</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="R3" s="2" t="s">
         <v>147</v>
@@ -29852,7 +29855,7 @@
       <c r="CN3" s="5"/>
       <c r="CO3" s="1"/>
       <c r="CQ3" s="1" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="CR3" s="1"/>
       <c r="CS3" s="1"/>

</xml_diff>

<commit_message>
- Detalles solucionados (07-05-2025)
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="ON" sheetId="1" state="visible" r:id="rId2"/>
@@ -29,6 +29,20 @@
     <author> </author>
   </authors>
   <commentList>
+    <comment ref="M2" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">Obligatorio</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="S2" authorId="0">
       <text>
         <r>
@@ -647,7 +661,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1465" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="331">
   <si>
     <t xml:space="preserve">Activo</t>
   </si>
@@ -1108,7 +1122,13 @@
     <t xml:space="preserve">Kran Kreen</t>
   </si>
   <si>
+    <t xml:space="preserve">HOTEL WPU</t>
+  </si>
+  <si>
     <t xml:space="preserve">TBC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCL</t>
   </si>
   <si>
     <t xml:space="preserve">ATO</t>
@@ -1175,9 +1195,6 @@
   </si>
   <si>
     <t xml:space="preserve">8:15 09:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HOTEL WPU</t>
   </si>
   <si>
     <t xml:space="preserve">Esta es una segunda prueba</t>
@@ -3359,12 +3376,8 @@
       <c r="AN3" s="47" t="s">
         <v>147</v>
       </c>
-      <c r="AO3" s="42" t="n">
-        <v>45660</v>
-      </c>
-      <c r="AP3" s="46" t="s">
-        <v>149</v>
-      </c>
+      <c r="AO3" s="42"/>
+      <c r="AP3" s="46"/>
       <c r="AQ3" s="40" t="s">
         <v>123</v>
       </c>
@@ -3383,9 +3396,7 @@
       <c r="AV3" s="40" t="s">
         <v>128</v>
       </c>
-      <c r="AW3" s="40" t="n">
-        <v>3</v>
-      </c>
+      <c r="AW3" s="40"/>
       <c r="AX3" s="40" t="s">
         <v>150</v>
       </c>
@@ -3401,7 +3412,9 @@
       <c r="BB3" s="40" t="s">
         <v>152</v>
       </c>
-      <c r="BC3" s="40"/>
+      <c r="BC3" s="40" t="s">
+        <v>153</v>
+      </c>
       <c r="BD3" s="42" t="n">
         <v>45671</v>
       </c>
@@ -3412,7 +3425,7 @@
         <v>151</v>
       </c>
       <c r="BG3" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BH3" s="40" t="s">
         <v>147</v>
@@ -3424,16 +3437,16 @@
         <v>152</v>
       </c>
       <c r="BM3" s="40" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="BN3" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BO3" s="40" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="BP3" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BQ3" s="42" t="n">
         <f aca="false">AL3</f>
@@ -3443,39 +3456,39 @@
         <v>0.0423611111111111</v>
       </c>
       <c r="BS3" s="40" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="BT3" s="40" t="s">
+        <v>157</v>
+      </c>
+      <c r="BU3" s="40" t="s">
         <v>155</v>
       </c>
-      <c r="BU3" s="40" t="s">
-        <v>135</v>
-      </c>
       <c r="BV3" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW3" s="42" t="n">
         <f aca="false">AO3</f>
-        <v>45660</v>
+        <v>0</v>
       </c>
       <c r="BX3" s="44" t="n">
         <v>0.0423611111111111</v>
       </c>
       <c r="BY3" s="40" t="s">
+        <v>147</v>
+      </c>
+      <c r="BZ3" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="BZ3" s="42" t="s">
-        <v>154</v>
-      </c>
       <c r="CA3" s="39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="CB3" s="39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="CC3" s="42" t="n">
         <f aca="false">AO3</f>
-        <v>45660</v>
+        <v>0</v>
       </c>
       <c r="CD3" s="44" t="n">
         <v>0.0423611111111111</v>
@@ -3508,7 +3521,7 @@
       <c r="DA3" s="42"/>
       <c r="DB3" s="40"/>
       <c r="DC3" s="51" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" s="51" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3541,20 +3554,20 @@
         <v>113</v>
       </c>
       <c r="K4" s="41" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="L4" s="41" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="M4" s="39"/>
       <c r="N4" s="41" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="O4" s="41" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="P4" s="40" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="Q4" s="43" t="n">
         <v>32524</v>
@@ -3568,31 +3581,31 @@
       <c r="T4" s="41"/>
       <c r="U4" s="40"/>
       <c r="V4" s="41" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="W4" s="42" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="X4" s="42" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="Y4" s="40" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="Z4" s="42" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="AA4" s="42" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="AB4" s="40" t="s">
+        <v>172</v>
+      </c>
+      <c r="AC4" s="42" t="s">
         <v>170</v>
       </c>
-      <c r="AC4" s="42" t="s">
-        <v>168</v>
-      </c>
       <c r="AD4" s="42" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="AE4" s="40" t="s">
         <v>147</v>
@@ -3604,7 +3617,7 @@
         <v>147</v>
       </c>
       <c r="AH4" s="41" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="AI4" s="42" t="n">
         <v>45660</v>
@@ -3613,7 +3626,7 @@
         <v>0.40625</v>
       </c>
       <c r="AK4" s="45" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="AL4" s="42" t="n">
         <v>45660</v>
@@ -3622,13 +3635,13 @@
         <v>149</v>
       </c>
       <c r="AN4" s="47" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="AO4" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP4" s="42" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="AQ4" s="40" t="s">
         <v>123</v>
@@ -3666,9 +3679,7 @@
       <c r="BB4" s="40" t="s">
         <v>152</v>
       </c>
-      <c r="BC4" s="40" t="s">
-        <v>176</v>
-      </c>
+      <c r="BC4" s="40"/>
       <c r="BD4" s="42" t="n">
         <v>45671</v>
       </c>
@@ -3679,7 +3690,7 @@
         <v>151</v>
       </c>
       <c r="BG4" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BH4" s="40" t="s">
         <v>147</v>
@@ -3694,13 +3705,13 @@
         <v>135</v>
       </c>
       <c r="BN4" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BO4" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP4" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BQ4" s="42" t="n">
         <f aca="false">AL4</f>
@@ -3713,13 +3724,13 @@
         <v>135</v>
       </c>
       <c r="BT4" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BU4" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV4" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW4" s="42" t="n">
         <f aca="false">AO4</f>
@@ -3729,16 +3740,16 @@
         <v>1.04236111111111</v>
       </c>
       <c r="BY4" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="BZ4" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="BZ4" s="42" t="s">
-        <v>154</v>
-      </c>
       <c r="CA4" s="39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="CB4" s="39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="CC4" s="42" t="n">
         <f aca="false">AO4</f>
@@ -3773,7 +3784,7 @@
       <c r="DA4" s="42"/>
       <c r="DB4" s="40"/>
       <c r="DC4" s="51" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" s="51" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3806,26 +3817,26 @@
         <v>113</v>
       </c>
       <c r="K5" s="41" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="L5" s="41" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="M5" s="39"/>
       <c r="N5" s="41" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="O5" s="41" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="P5" s="40" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="Q5" s="43" t="n">
         <v>32346</v>
       </c>
       <c r="R5" s="41" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="S5" s="41" t="s">
         <v>120</v>
@@ -3833,13 +3844,13 @@
       <c r="T5" s="41"/>
       <c r="U5" s="40"/>
       <c r="V5" s="41" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="W5" s="42" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="X5" s="42" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="Y5" s="40" t="s">
         <v>147</v>
@@ -3869,7 +3880,7 @@
         <v>147</v>
       </c>
       <c r="AH5" s="41" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="AI5" s="42" t="n">
         <v>45661</v>
@@ -3878,22 +3889,22 @@
         <v>0.472222222222222</v>
       </c>
       <c r="AK5" s="45" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AL5" s="42" t="n">
         <v>45661</v>
       </c>
       <c r="AM5" s="46" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="AN5" s="47" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="AO5" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP5" s="40" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="AQ5" s="40" t="s">
         <v>123</v>
@@ -3926,13 +3937,13 @@
         <v>45662</v>
       </c>
       <c r="BA5" s="40" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="BB5" s="40" t="s">
         <v>152</v>
       </c>
       <c r="BC5" s="40" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="BD5" s="42" t="n">
         <v>45671</v>
@@ -3944,7 +3955,7 @@
         <v>151</v>
       </c>
       <c r="BG5" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BH5" s="40" t="s">
         <v>147</v>
@@ -3959,13 +3970,13 @@
         <v>135</v>
       </c>
       <c r="BN5" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BO5" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP5" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BQ5" s="42" t="n">
         <f aca="false">AL5</f>
@@ -3978,13 +3989,13 @@
         <v>135</v>
       </c>
       <c r="BT5" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BU5" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV5" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW5" s="42" t="n">
         <f aca="false">AO5</f>
@@ -3994,16 +4005,16 @@
         <v>2.04236111111111</v>
       </c>
       <c r="BY5" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="BZ5" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="BZ5" s="42" t="s">
-        <v>154</v>
-      </c>
       <c r="CA5" s="39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="CB5" s="39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="CC5" s="42" t="n">
         <f aca="false">AO5</f>
@@ -4070,20 +4081,20 @@
         <v>113</v>
       </c>
       <c r="K6" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="L6" s="41" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="M6" s="39"/>
       <c r="N6" s="41" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="O6" s="41" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P6" s="40" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="Q6" s="43" t="n">
         <v>30193</v>
@@ -4095,22 +4106,22 @@
       <c r="T6" s="41"/>
       <c r="U6" s="40"/>
       <c r="V6" s="41" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="W6" s="42" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="X6" s="42" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="Y6" s="40" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="Z6" s="42" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="AA6" s="42" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="AB6" s="40" t="s">
         <v>147</v>
@@ -4140,22 +4151,22 @@
         <v>0.388888888888889</v>
       </c>
       <c r="AK6" s="45" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AL6" s="42" t="n">
         <v>45661</v>
       </c>
       <c r="AM6" s="46" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="AN6" s="47" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="AO6" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP6" s="40" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="AQ6" s="40" t="s">
         <v>123</v>
@@ -4188,13 +4199,13 @@
         <v>45662</v>
       </c>
       <c r="BA6" s="40" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="BB6" s="40" t="s">
         <v>152</v>
       </c>
       <c r="BC6" s="40" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="BD6" s="42" t="n">
         <v>45671</v>
@@ -4206,7 +4217,7 @@
         <v>151</v>
       </c>
       <c r="BG6" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BH6" s="40" t="s">
         <v>147</v>
@@ -4221,13 +4232,13 @@
         <v>135</v>
       </c>
       <c r="BN6" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BO6" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP6" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BQ6" s="42" t="n">
         <f aca="false">AL6</f>
@@ -4240,13 +4251,13 @@
         <v>135</v>
       </c>
       <c r="BT6" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BU6" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV6" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW6" s="42" t="n">
         <f aca="false">AO6</f>
@@ -4256,16 +4267,16 @@
         <v>3.04236111111111</v>
       </c>
       <c r="BY6" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="BZ6" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="BZ6" s="42" t="s">
-        <v>154</v>
-      </c>
       <c r="CA6" s="39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="CB6" s="39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="CC6" s="42" t="n">
         <f aca="false">AO6</f>
@@ -4330,51 +4341,51 @@
         <v>113</v>
       </c>
       <c r="K7" s="41" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L7" s="41" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="M7" s="39"/>
       <c r="N7" s="41" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="O7" s="41" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="P7" s="40" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="Q7" s="43" t="n">
         <v>36383</v>
       </c>
       <c r="R7" s="41" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="S7" s="41" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="T7" s="41" t="s">
         <v>120</v>
       </c>
       <c r="U7" s="40"/>
       <c r="V7" s="41" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="W7" s="42" t="n">
         <v>45661</v>
       </c>
       <c r="X7" s="42" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="Y7" s="40" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="Z7" s="42" t="n">
         <v>45661</v>
       </c>
       <c r="AA7" s="42" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AB7" s="40" t="s">
         <v>147</v>
@@ -4395,7 +4406,7 @@
         <v>147</v>
       </c>
       <c r="AH7" s="41" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="AI7" s="42" t="n">
         <v>45661</v>
@@ -4404,22 +4415,22 @@
         <v>0.451388888888889</v>
       </c>
       <c r="AK7" s="45" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AL7" s="42" t="n">
         <v>45661</v>
       </c>
       <c r="AM7" s="46" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="AN7" s="47" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="AO7" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP7" s="40" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="AQ7" s="40" t="s">
         <v>123</v>
@@ -4458,7 +4469,7 @@
         <v>152</v>
       </c>
       <c r="BC7" s="40" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="BD7" s="42" t="n">
         <v>45671</v>
@@ -4470,7 +4481,7 @@
         <v>151</v>
       </c>
       <c r="BG7" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BH7" s="40" t="s">
         <v>147</v>
@@ -4485,13 +4496,13 @@
         <v>135</v>
       </c>
       <c r="BN7" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BO7" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP7" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BQ7" s="42" t="n">
         <f aca="false">AL7</f>
@@ -4504,13 +4515,13 @@
         <v>135</v>
       </c>
       <c r="BT7" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BU7" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV7" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW7" s="42" t="n">
         <f aca="false">AO7</f>
@@ -4520,16 +4531,16 @@
         <v>4.04236111111111</v>
       </c>
       <c r="BY7" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="BZ7" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="BZ7" s="42" t="s">
-        <v>154</v>
-      </c>
       <c r="CA7" s="39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="CB7" s="39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="CC7" s="42" t="n">
         <f aca="false">AO7</f>
@@ -4596,26 +4607,26 @@
         <v>113</v>
       </c>
       <c r="K8" s="41" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="L8" s="41" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="M8" s="39"/>
       <c r="N8" s="41" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="O8" s="41" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="P8" s="40" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="Q8" s="43" t="n">
         <v>29208</v>
       </c>
       <c r="R8" s="41" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="S8" s="41" t="s">
         <v>120</v>
@@ -4623,31 +4634,31 @@
       <c r="T8" s="41"/>
       <c r="U8" s="40"/>
       <c r="V8" s="52" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="W8" s="53" t="n">
         <v>45667</v>
       </c>
       <c r="X8" s="53" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Y8" s="54" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="Z8" s="53" t="n">
         <v>45668</v>
       </c>
       <c r="AA8" s="53" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AB8" s="54" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AC8" s="53" t="n">
         <v>45668</v>
       </c>
       <c r="AD8" s="53" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AE8" s="40" t="s">
         <v>147</v>
@@ -4659,7 +4670,7 @@
         <v>147</v>
       </c>
       <c r="AH8" s="41" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="AI8" s="42" t="n">
         <v>45661</v>
@@ -4668,22 +4679,22 @@
         <v>0.451388888888889</v>
       </c>
       <c r="AK8" s="45" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AL8" s="42" t="n">
         <v>45661</v>
       </c>
       <c r="AM8" s="46" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="AN8" s="47" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="AO8" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP8" s="40" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="AQ8" s="40" t="s">
         <v>123</v>
@@ -4716,13 +4727,13 @@
         <v>45662</v>
       </c>
       <c r="BA8" s="40" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="BB8" s="40" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="BC8" s="40" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="BD8" s="42" t="n">
         <v>45671</v>
@@ -4734,7 +4745,7 @@
         <v>151</v>
       </c>
       <c r="BG8" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BH8" s="40" t="s">
         <v>147</v>
@@ -4743,19 +4754,19 @@
       <c r="BJ8" s="43"/>
       <c r="BK8" s="40"/>
       <c r="BL8" s="40" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="BM8" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN8" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BO8" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP8" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BQ8" s="42" t="n">
         <f aca="false">AL8</f>
@@ -4768,13 +4779,13 @@
         <v>135</v>
       </c>
       <c r="BT8" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BU8" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV8" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW8" s="42" t="n">
         <f aca="false">AO8</f>
@@ -4784,16 +4795,16 @@
         <v>5.04236111111111</v>
       </c>
       <c r="BY8" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="BZ8" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="BZ8" s="42" t="s">
-        <v>154</v>
-      </c>
       <c r="CA8" s="39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="CB8" s="39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="CC8" s="42" t="n">
         <f aca="false">AO8</f>
@@ -4853,26 +4864,26 @@
         <v>113</v>
       </c>
       <c r="K9" s="41" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="L9" s="41" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="M9" s="39"/>
       <c r="N9" s="41" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="O9" s="41" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="P9" s="40" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="Q9" s="43" t="n">
         <v>33062</v>
       </c>
       <c r="R9" s="41" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="S9" s="41" t="s">
         <v>120</v>
@@ -4880,31 +4891,31 @@
       <c r="T9" s="41"/>
       <c r="U9" s="40"/>
       <c r="V9" s="41" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="W9" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X9" s="42" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Y9" s="40" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="Z9" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA9" s="42" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AB9" s="40" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AC9" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AD9" s="42" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AE9" s="40" t="s">
         <v>147</v>
@@ -4916,7 +4927,7 @@
         <v>147</v>
       </c>
       <c r="AH9" s="41" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="AI9" s="42" t="n">
         <v>45661</v>
@@ -4925,22 +4936,22 @@
         <v>0.409722222222222</v>
       </c>
       <c r="AK9" s="45" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="AL9" s="42" t="n">
         <v>45661</v>
       </c>
       <c r="AM9" s="46" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="AN9" s="47" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="AO9" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP9" s="40" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="AQ9" s="40" t="s">
         <v>123</v>
@@ -4979,7 +4990,7 @@
         <v>152</v>
       </c>
       <c r="BC9" s="40" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="BD9" s="42" t="n">
         <v>45671</v>
@@ -4991,7 +5002,7 @@
         <v>151</v>
       </c>
       <c r="BG9" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BH9" s="40" t="s">
         <v>147</v>
@@ -5006,13 +5017,13 @@
         <v>135</v>
       </c>
       <c r="BN9" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BO9" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP9" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BQ9" s="42" t="n">
         <f aca="false">AL9</f>
@@ -5025,13 +5036,13 @@
         <v>135</v>
       </c>
       <c r="BT9" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BU9" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV9" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW9" s="42" t="n">
         <f aca="false">AO9</f>
@@ -5041,16 +5052,16 @@
         <v>6.04236111111111</v>
       </c>
       <c r="BY9" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="BZ9" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="BZ9" s="42" t="s">
-        <v>154</v>
-      </c>
       <c r="CA9" s="39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="CB9" s="39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="CC9" s="42" t="n">
         <f aca="false">AO9</f>
@@ -5088,7 +5099,7 @@
         <v>108</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D10" s="42"/>
       <c r="E10" s="42" t="n">
@@ -5098,7 +5109,7 @@
         <v>45663</v>
       </c>
       <c r="G10" s="40" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H10" s="40" t="s">
         <v>142</v>
@@ -5110,20 +5121,20 @@
         <v>113</v>
       </c>
       <c r="K10" s="41" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="L10" s="41" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="M10" s="39"/>
       <c r="N10" s="41" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="O10" s="41" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="P10" s="40" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="Q10" s="43" t="n">
         <v>33794</v>
@@ -5137,31 +5148,31 @@
       <c r="T10" s="41"/>
       <c r="U10" s="40"/>
       <c r="V10" s="41" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="W10" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X10" s="42" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Y10" s="40" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="Z10" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA10" s="42" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AB10" s="40" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AC10" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AD10" s="42" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AE10" s="40" t="s">
         <v>147</v>
@@ -5173,7 +5184,7 @@
         <v>147</v>
       </c>
       <c r="AH10" s="41" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI10" s="42" t="n">
         <v>45662</v>
@@ -5182,18 +5193,18 @@
         <v>0.40625</v>
       </c>
       <c r="AK10" s="45" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="AL10" s="42" t="n">
         <v>45662</v>
       </c>
       <c r="AM10" s="46" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="AN10" s="47" t="s">
         <v>147</v>
       </c>
-      <c r="AO10" s="40"/>
+      <c r="AO10" s="42"/>
       <c r="AP10" s="40"/>
       <c r="AQ10" s="40" t="s">
         <v>123</v>
@@ -5226,13 +5237,13 @@
         <v>45663</v>
       </c>
       <c r="BA10" s="40" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="BB10" s="40" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="BC10" s="40" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="BD10" s="42" t="n">
         <v>45671</v>
@@ -5244,7 +5255,7 @@
         <v>151</v>
       </c>
       <c r="BG10" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BH10" s="40" t="s">
         <v>147</v>
@@ -5253,19 +5264,19 @@
       <c r="BJ10" s="43"/>
       <c r="BK10" s="40"/>
       <c r="BL10" s="40" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="BM10" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN10" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BO10" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP10" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BQ10" s="42" t="n">
         <f aca="false">AL10</f>
@@ -5278,13 +5289,13 @@
         <v>135</v>
       </c>
       <c r="BT10" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BU10" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV10" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW10" s="42" t="n">
         <f aca="false">AO10</f>
@@ -5294,16 +5305,16 @@
         <v>7.04236111111111</v>
       </c>
       <c r="BY10" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="BZ10" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="BZ10" s="42" t="s">
-        <v>154</v>
-      </c>
       <c r="CA10" s="39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="CB10" s="39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="CC10" s="55" t="n">
         <v>36892</v>
@@ -5362,20 +5373,20 @@
         <v>113</v>
       </c>
       <c r="K11" s="41" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="L11" s="41" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="M11" s="39"/>
       <c r="N11" s="41" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="O11" s="41" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="P11" s="40" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="Q11" s="43" t="n">
         <v>33386</v>
@@ -5389,31 +5400,31 @@
       <c r="T11" s="41"/>
       <c r="U11" s="40"/>
       <c r="V11" s="41" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="W11" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X11" s="42" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="Y11" s="40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="Z11" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA11" s="42" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="AB11" s="40" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="AC11" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AD11" s="42" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="AE11" s="40" t="s">
         <v>147</v>
@@ -5425,7 +5436,7 @@
         <v>147</v>
       </c>
       <c r="AH11" s="41" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="AI11" s="42" t="n">
         <v>45665</v>
@@ -5434,22 +5445,22 @@
         <v>0.354166666666667</v>
       </c>
       <c r="AK11" s="45" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="AL11" s="42" t="n">
         <v>45665</v>
       </c>
       <c r="AM11" s="46" t="s">
+        <v>249</v>
+      </c>
+      <c r="AN11" s="57" t="s">
         <v>248</v>
-      </c>
-      <c r="AN11" s="57" t="s">
-        <v>247</v>
       </c>
       <c r="AO11" s="42" t="n">
         <v>45665</v>
       </c>
       <c r="AP11" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="AQ11" s="40" t="s">
         <v>123</v>
@@ -5482,13 +5493,13 @@
         <v>45663</v>
       </c>
       <c r="BA11" s="40" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="BB11" s="40" t="s">
+        <v>154</v>
+      </c>
+      <c r="BC11" s="40" t="s">
         <v>153</v>
-      </c>
-      <c r="BC11" s="40" t="s">
-        <v>176</v>
       </c>
       <c r="BD11" s="42" t="n">
         <v>45671</v>
@@ -5500,7 +5511,7 @@
         <v>151</v>
       </c>
       <c r="BG11" s="40" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="BH11" s="40" t="s">
         <v>147</v>
@@ -5564,7 +5575,7 @@
         <v>108</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D12" s="42"/>
       <c r="E12" s="42" t="n">
@@ -5586,58 +5597,58 @@
         <v>113</v>
       </c>
       <c r="K12" s="41" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="L12" s="41" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="M12" s="39"/>
       <c r="N12" s="41" t="s">
         <v>145</v>
       </c>
       <c r="O12" s="41" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="P12" s="40" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="Q12" s="43" t="n">
         <v>35988</v>
       </c>
       <c r="R12" s="41" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="S12" s="41" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="T12" s="41"/>
       <c r="U12" s="40"/>
       <c r="V12" s="41" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="W12" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X12" s="42" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="Y12" s="40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="Z12" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA12" s="42" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="AB12" s="40" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="AC12" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AD12" s="42" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="AE12" s="40" t="s">
         <v>147</v>
@@ -5649,7 +5660,7 @@
         <v>147</v>
       </c>
       <c r="AH12" s="41" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AI12" s="42" t="n">
         <v>45668</v>
@@ -5658,22 +5669,22 @@
         <v>0.732638888888889</v>
       </c>
       <c r="AK12" s="45" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="AL12" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM12" s="46" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="AN12" s="47" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="AO12" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP12" s="40" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AQ12" s="40" t="s">
         <v>123</v>
@@ -5712,7 +5723,7 @@
         <v>152</v>
       </c>
       <c r="BC12" s="40" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="BD12" s="42" t="n">
         <v>45671</v>
@@ -5724,7 +5735,7 @@
         <v>151</v>
       </c>
       <c r="BG12" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BH12" s="40" t="s">
         <v>147</v>
@@ -5739,13 +5750,13 @@
         <v>135</v>
       </c>
       <c r="BN12" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BO12" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP12" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BQ12" s="42" t="n">
         <f aca="false">AL12</f>
@@ -5758,13 +5769,13 @@
         <v>135</v>
       </c>
       <c r="BT12" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BU12" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV12" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW12" s="42" t="n">
         <f aca="false">AO12</f>
@@ -5774,16 +5785,16 @@
         <v>9.04236111111111</v>
       </c>
       <c r="BY12" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="BZ12" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="BZ12" s="42" t="s">
-        <v>154</v>
-      </c>
       <c r="CA12" s="39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="CB12" s="39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="CC12" s="42" t="n">
         <f aca="false">AO12</f>
@@ -5821,7 +5832,7 @@
         <v>108</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D13" s="42"/>
       <c r="E13" s="42" t="n">
@@ -5843,26 +5854,26 @@
         <v>113</v>
       </c>
       <c r="K13" s="41" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="L13" s="41" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="M13" s="39"/>
       <c r="N13" s="41" t="s">
         <v>145</v>
       </c>
       <c r="O13" s="41" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="P13" s="40" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="Q13" s="43" t="n">
         <v>29371</v>
       </c>
       <c r="R13" s="41" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="S13" s="41" t="s">
         <v>120</v>
@@ -5870,31 +5881,31 @@
       <c r="T13" s="41"/>
       <c r="U13" s="40"/>
       <c r="V13" s="41" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="W13" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X13" s="42" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Y13" s="40" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="Z13" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA13" s="42" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AB13" s="40" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AC13" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AD13" s="42" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AE13" s="40" t="s">
         <v>147</v>
@@ -5906,7 +5917,7 @@
         <v>147</v>
       </c>
       <c r="AH13" s="41" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AI13" s="42" t="n">
         <v>45668</v>
@@ -5915,22 +5926,22 @@
         <v>0.732638888888889</v>
       </c>
       <c r="AK13" s="45" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="AL13" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM13" s="46" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="AN13" s="47" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="AO13" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP13" s="40" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AQ13" s="40" t="s">
         <v>123</v>
@@ -5969,7 +5980,7 @@
         <v>152</v>
       </c>
       <c r="BC13" s="40" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="BD13" s="42" t="n">
         <v>45671</v>
@@ -5981,7 +5992,7 @@
         <v>151</v>
       </c>
       <c r="BG13" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BH13" s="40" t="s">
         <v>147</v>
@@ -5996,13 +6007,13 @@
         <v>135</v>
       </c>
       <c r="BN13" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BO13" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP13" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BQ13" s="42" t="n">
         <f aca="false">AL13</f>
@@ -6015,13 +6026,13 @@
         <v>135</v>
       </c>
       <c r="BT13" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BU13" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV13" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW13" s="42" t="n">
         <f aca="false">AO13</f>
@@ -6031,16 +6042,16 @@
         <v>10.0423611111111</v>
       </c>
       <c r="BY13" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="BZ13" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="BZ13" s="42" t="s">
-        <v>154</v>
-      </c>
       <c r="CA13" s="39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="CB13" s="39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="CC13" s="42" t="n">
         <f aca="false">AO13</f>
@@ -6078,7 +6089,7 @@
         <v>108</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D14" s="42"/>
       <c r="E14" s="42" t="n">
@@ -6100,26 +6111,26 @@
         <v>113</v>
       </c>
       <c r="K14" s="41" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="L14" s="41" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="M14" s="39"/>
       <c r="N14" s="41" t="s">
         <v>145</v>
       </c>
       <c r="O14" s="41" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="P14" s="40" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="Q14" s="43" t="n">
         <v>32894</v>
       </c>
       <c r="R14" s="41" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="S14" s="41" t="s">
         <v>120</v>
@@ -6127,31 +6138,31 @@
       <c r="T14" s="41"/>
       <c r="U14" s="40"/>
       <c r="V14" s="41" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="W14" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X14" s="42" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="Y14" s="40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="Z14" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA14" s="42" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="AB14" s="40" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="AC14" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AD14" s="42" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="AE14" s="40" t="s">
         <v>147</v>
@@ -6163,7 +6174,7 @@
         <v>147</v>
       </c>
       <c r="AH14" s="41" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="AI14" s="42" t="n">
         <v>45668</v>
@@ -6172,22 +6183,22 @@
         <v>0.590277777777778</v>
       </c>
       <c r="AK14" s="45" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="AL14" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM14" s="46" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AN14" s="47" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="AO14" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP14" s="40" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AQ14" s="40" t="s">
         <v>123</v>
@@ -6226,7 +6237,7 @@
         <v>152</v>
       </c>
       <c r="BC14" s="40" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="BD14" s="42" t="n">
         <v>45671</v>
@@ -6238,7 +6249,7 @@
         <v>151</v>
       </c>
       <c r="BG14" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BH14" s="40" t="s">
         <v>147</v>
@@ -6253,13 +6264,13 @@
         <v>135</v>
       </c>
       <c r="BN14" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BO14" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP14" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BQ14" s="42" t="n">
         <f aca="false">AL14</f>
@@ -6272,13 +6283,13 @@
         <v>135</v>
       </c>
       <c r="BT14" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BU14" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV14" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW14" s="42" t="n">
         <f aca="false">AO14</f>
@@ -6288,16 +6299,16 @@
         <v>11.0423611111111</v>
       </c>
       <c r="BY14" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="BZ14" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="BZ14" s="42" t="s">
-        <v>154</v>
-      </c>
       <c r="CA14" s="39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="CB14" s="39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="CC14" s="42" t="n">
         <f aca="false">AO14</f>
@@ -6335,7 +6346,7 @@
         <v>108</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D15" s="42"/>
       <c r="E15" s="42" t="n">
@@ -6357,26 +6368,26 @@
         <v>113</v>
       </c>
       <c r="K15" s="41" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="L15" s="41" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="M15" s="39"/>
       <c r="N15" s="41" t="s">
         <v>145</v>
       </c>
       <c r="O15" s="41" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="P15" s="40" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="Q15" s="43" t="n">
         <v>32113</v>
       </c>
       <c r="R15" s="41" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="S15" s="41" t="s">
         <v>120</v>
@@ -6384,31 +6395,31 @@
       <c r="T15" s="41"/>
       <c r="U15" s="40"/>
       <c r="V15" s="41" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="W15" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X15" s="42" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Y15" s="40" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="Z15" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA15" s="42" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AB15" s="40" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AC15" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AD15" s="42" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AE15" s="40" t="s">
         <v>147</v>
@@ -6420,7 +6431,7 @@
         <v>147</v>
       </c>
       <c r="AH15" s="41" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="AI15" s="42" t="n">
         <v>45668</v>
@@ -6429,22 +6440,22 @@
         <v>0.590277777777778</v>
       </c>
       <c r="AK15" s="45" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="AL15" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM15" s="46" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AN15" s="47" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="AO15" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP15" s="40" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AQ15" s="40" t="s">
         <v>123</v>
@@ -6483,7 +6494,7 @@
         <v>152</v>
       </c>
       <c r="BC15" s="40" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="BD15" s="42" t="n">
         <v>45671</v>
@@ -6495,7 +6506,7 @@
         <v>151</v>
       </c>
       <c r="BG15" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BH15" s="40" t="s">
         <v>147</v>
@@ -6510,13 +6521,13 @@
         <v>135</v>
       </c>
       <c r="BN15" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BO15" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP15" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BQ15" s="42" t="n">
         <f aca="false">AL15</f>
@@ -6529,13 +6540,13 @@
         <v>135</v>
       </c>
       <c r="BT15" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BU15" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV15" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW15" s="42" t="n">
         <f aca="false">AO15</f>
@@ -6545,16 +6556,16 @@
         <v>12.0423611111111</v>
       </c>
       <c r="BY15" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="BZ15" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="BZ15" s="42" t="s">
-        <v>154</v>
-      </c>
       <c r="CA15" s="39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="CB15" s="39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="CC15" s="42" t="n">
         <f aca="false">AO15</f>
@@ -6592,7 +6603,7 @@
         <v>108</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D16" s="42"/>
       <c r="E16" s="42" t="n">
@@ -6614,58 +6625,58 @@
         <v>113</v>
       </c>
       <c r="K16" s="41" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="L16" s="41" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="M16" s="39"/>
       <c r="N16" s="41" t="s">
         <v>145</v>
       </c>
       <c r="O16" s="41" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="P16" s="40" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="Q16" s="43" t="n">
         <v>35754</v>
       </c>
       <c r="R16" s="41" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="S16" s="41" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="T16" s="41"/>
       <c r="U16" s="40"/>
       <c r="V16" s="41" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="W16" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X16" s="42" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Y16" s="40" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="Z16" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA16" s="42" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AB16" s="40" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AC16" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AD16" s="42" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AE16" s="40" t="s">
         <v>147</v>
@@ -6677,7 +6688,7 @@
         <v>147</v>
       </c>
       <c r="AH16" s="41" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AI16" s="42" t="n">
         <v>45668</v>
@@ -6686,22 +6697,22 @@
         <v>0.732638888888889</v>
       </c>
       <c r="AK16" s="45" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="AL16" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM16" s="46" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="AN16" s="47" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="AO16" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP16" s="40" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AQ16" s="40" t="s">
         <v>123</v>
@@ -6737,10 +6748,10 @@
         <v>151</v>
       </c>
       <c r="BB16" s="40" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="BC16" s="40" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="BD16" s="42" t="n">
         <v>45671</v>
@@ -6752,7 +6763,7 @@
         <v>151</v>
       </c>
       <c r="BG16" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BH16" s="40" t="s">
         <v>147</v>
@@ -6761,19 +6772,19 @@
       <c r="BJ16" s="43"/>
       <c r="BK16" s="40"/>
       <c r="BL16" s="40" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="BM16" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN16" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BO16" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP16" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BQ16" s="42" t="n">
         <f aca="false">AL16</f>
@@ -6786,13 +6797,13 @@
         <v>135</v>
       </c>
       <c r="BT16" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BU16" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV16" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW16" s="42" t="n">
         <f aca="false">AO16</f>
@@ -6802,16 +6813,16 @@
         <v>13.0423611111111</v>
       </c>
       <c r="BY16" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="BZ16" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="BZ16" s="42" t="s">
-        <v>154</v>
-      </c>
       <c r="CA16" s="39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="CB16" s="39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="CC16" s="42" t="n">
         <f aca="false">AO16</f>
@@ -6849,7 +6860,7 @@
         <v>108</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D17" s="42"/>
       <c r="E17" s="42" t="n">
@@ -6871,26 +6882,26 @@
         <v>113</v>
       </c>
       <c r="K17" s="41" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="L17" s="41" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="M17" s="39"/>
       <c r="N17" s="41" t="s">
         <v>145</v>
       </c>
       <c r="O17" s="41" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="P17" s="40" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="Q17" s="43" t="n">
         <v>33264</v>
       </c>
       <c r="R17" s="41" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="S17" s="41" t="s">
         <v>120</v>
@@ -6898,22 +6909,22 @@
       <c r="T17" s="41"/>
       <c r="U17" s="40"/>
       <c r="V17" s="41" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="W17" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X17" s="42" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="Y17" s="40" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="Z17" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA17" s="42" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="AB17" s="40" t="s">
         <v>147</v>
@@ -6934,7 +6945,7 @@
         <v>147</v>
       </c>
       <c r="AH17" s="41" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="AI17" s="42" t="n">
         <v>45668</v>
@@ -6943,22 +6954,22 @@
         <v>0.590277777777778</v>
       </c>
       <c r="AK17" s="45" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="AL17" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM17" s="46" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AN17" s="47" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="AO17" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP17" s="40" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AQ17" s="40" t="s">
         <v>123</v>
@@ -6997,7 +7008,7 @@
         <v>152</v>
       </c>
       <c r="BC17" s="40" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="BD17" s="42" t="n">
         <v>45671</v>
@@ -7009,7 +7020,7 @@
         <v>151</v>
       </c>
       <c r="BG17" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BH17" s="40" t="s">
         <v>147</v>
@@ -7024,13 +7035,13 @@
         <v>135</v>
       </c>
       <c r="BN17" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BO17" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP17" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BQ17" s="42" t="n">
         <f aca="false">AL17</f>
@@ -7043,13 +7054,13 @@
         <v>135</v>
       </c>
       <c r="BT17" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BU17" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV17" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW17" s="42" t="n">
         <f aca="false">AO17</f>
@@ -7059,16 +7070,16 @@
         <v>14.0423611111111</v>
       </c>
       <c r="BY17" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="BZ17" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="BZ17" s="42" t="s">
-        <v>154</v>
-      </c>
       <c r="CA17" s="39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="CB17" s="39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="CC17" s="42" t="n">
         <f aca="false">AO17</f>
@@ -7106,7 +7117,7 @@
         <v>108</v>
       </c>
       <c r="C18" s="41" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D18" s="42"/>
       <c r="E18" s="42" t="n">
@@ -7128,58 +7139,58 @@
         <v>113</v>
       </c>
       <c r="K18" s="41" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L18" s="41" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="M18" s="39"/>
       <c r="N18" s="41" t="s">
         <v>145</v>
       </c>
       <c r="O18" s="41" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="P18" s="40" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="Q18" s="43" t="n">
         <v>28156</v>
       </c>
       <c r="R18" s="41" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="S18" s="41" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="T18" s="41"/>
       <c r="U18" s="40"/>
       <c r="V18" s="41" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="W18" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X18" s="42" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="Y18" s="40" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="Z18" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA18" s="42" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AB18" s="40" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AC18" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AD18" s="42" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AE18" s="40" t="s">
         <v>147</v>
@@ -7191,7 +7202,7 @@
         <v>147</v>
       </c>
       <c r="AH18" s="41" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AI18" s="42" t="n">
         <v>45668</v>
@@ -7200,22 +7211,22 @@
         <v>0.732638888888889</v>
       </c>
       <c r="AK18" s="45" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="AL18" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM18" s="46" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="AN18" s="47" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="AO18" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP18" s="40" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AQ18" s="40" t="s">
         <v>123</v>
@@ -7251,10 +7262,10 @@
         <v>151</v>
       </c>
       <c r="BB18" s="40" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="BC18" s="40" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="BD18" s="42" t="n">
         <v>45671</v>
@@ -7266,7 +7277,7 @@
         <v>151</v>
       </c>
       <c r="BG18" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BH18" s="40" t="s">
         <v>147</v>
@@ -7275,19 +7286,19 @@
       <c r="BJ18" s="43"/>
       <c r="BK18" s="40"/>
       <c r="BL18" s="40" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="BM18" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN18" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BO18" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP18" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BQ18" s="42" t="n">
         <f aca="false">AL18</f>
@@ -7300,13 +7311,13 @@
         <v>135</v>
       </c>
       <c r="BT18" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BU18" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV18" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW18" s="42" t="n">
         <f aca="false">AO18</f>
@@ -7316,16 +7327,16 @@
         <v>15.0423611111111</v>
       </c>
       <c r="BY18" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="BZ18" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="BZ18" s="42" t="s">
-        <v>154</v>
-      </c>
       <c r="CA18" s="39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="CB18" s="39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="CC18" s="42" t="n">
         <f aca="false">AO18</f>
@@ -7363,7 +7374,7 @@
         <v>108</v>
       </c>
       <c r="C19" s="58" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D19" s="59"/>
       <c r="E19" s="42" t="n">
@@ -7385,57 +7396,57 @@
         <v>113</v>
       </c>
       <c r="K19" s="58" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="L19" s="58" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="N19" s="58" t="s">
         <v>145</v>
       </c>
       <c r="O19" s="58" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="P19" s="48" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="Q19" s="43" t="n">
         <v>33314</v>
       </c>
       <c r="R19" s="58" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="S19" s="58" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="T19" s="58"/>
       <c r="U19" s="48"/>
       <c r="V19" s="58" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="W19" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="X19" s="59" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="Y19" s="48" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="Z19" s="59" t="n">
         <v>45669</v>
       </c>
       <c r="AA19" s="59" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AB19" s="48" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AC19" s="59" t="n">
         <v>45669</v>
       </c>
       <c r="AD19" s="59" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AE19" s="48" t="s">
         <v>147</v>
@@ -7447,7 +7458,7 @@
         <v>147</v>
       </c>
       <c r="AH19" s="58" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AI19" s="59" t="n">
         <v>45668</v>
@@ -7456,22 +7467,22 @@
         <v>0.732638888888889</v>
       </c>
       <c r="AK19" s="61" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="AL19" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM19" s="62" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="AN19" s="47" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="AO19" s="59" t="n">
         <v>45670</v>
       </c>
       <c r="AP19" s="40" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AQ19" s="40" t="s">
         <v>123</v>
@@ -7507,10 +7518,10 @@
         <v>151</v>
       </c>
       <c r="BB19" s="48" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="BC19" s="40" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="BD19" s="42" t="n">
         <v>45671</v>
@@ -7522,7 +7533,7 @@
         <v>151</v>
       </c>
       <c r="BG19" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BH19" s="48" t="s">
         <v>147</v>
@@ -7531,19 +7542,19 @@
       <c r="BJ19" s="60"/>
       <c r="BK19" s="48"/>
       <c r="BL19" s="48" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="BM19" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN19" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BO19" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP19" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BQ19" s="42" t="n">
         <f aca="false">AL19</f>
@@ -7556,13 +7567,13 @@
         <v>135</v>
       </c>
       <c r="BT19" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BU19" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV19" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW19" s="42" t="n">
         <f aca="false">AO19</f>
@@ -7572,16 +7583,16 @@
         <v>16.0423611111111</v>
       </c>
       <c r="BY19" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="BZ19" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="BZ19" s="42" t="s">
-        <v>154</v>
-      </c>
       <c r="CA19" s="39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="CB19" s="39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="CC19" s="42" t="n">
         <f aca="false">AO19</f>
@@ -7616,7 +7627,7 @@
         <v>108</v>
       </c>
       <c r="C20" s="58" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D20" s="59"/>
       <c r="E20" s="42" t="n">
@@ -7638,19 +7649,19 @@
         <v>113</v>
       </c>
       <c r="K20" s="58" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L20" s="58" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="N20" s="58" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="O20" s="58" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="P20" s="48" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="Q20" s="43" t="n">
         <v>33003</v>
@@ -7662,31 +7673,31 @@
       <c r="T20" s="58"/>
       <c r="U20" s="48"/>
       <c r="V20" s="58" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="W20" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="X20" s="59" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="Y20" s="48" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="Z20" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="AA20" s="59" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="AB20" s="48" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="AC20" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="AD20" s="59" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="AE20" s="48" t="s">
         <v>147</v>
@@ -7698,7 +7709,7 @@
         <v>147</v>
       </c>
       <c r="AH20" s="58" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="AI20" s="59" t="n">
         <v>45668</v>
@@ -7707,22 +7718,22 @@
         <v>0.225694444444444</v>
       </c>
       <c r="AK20" s="61" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="AL20" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM20" s="62" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="AN20" s="47" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="AO20" s="59" t="n">
         <v>45670</v>
       </c>
       <c r="AP20" s="40" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AQ20" s="40" t="s">
         <v>123</v>
@@ -7761,7 +7772,7 @@
         <v>152</v>
       </c>
       <c r="BC20" s="40" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="BD20" s="42" t="n">
         <v>45671</v>
@@ -7773,7 +7784,7 @@
         <v>151</v>
       </c>
       <c r="BG20" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BH20" s="48" t="s">
         <v>147</v>
@@ -7788,13 +7799,13 @@
         <v>135</v>
       </c>
       <c r="BN20" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BO20" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP20" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BQ20" s="42" t="n">
         <f aca="false">AL20</f>
@@ -7807,13 +7818,13 @@
         <v>135</v>
       </c>
       <c r="BT20" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BU20" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV20" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW20" s="42" t="n">
         <f aca="false">AO20</f>
@@ -7823,16 +7834,16 @@
         <v>17.0423611111111</v>
       </c>
       <c r="BY20" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="BZ20" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="BZ20" s="42" t="s">
-        <v>154</v>
-      </c>
       <c r="CA20" s="39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="CB20" s="39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="CC20" s="42" t="n">
         <f aca="false">AO20</f>
@@ -7867,7 +7878,7 @@
         <v>108</v>
       </c>
       <c r="C21" s="58" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D21" s="59"/>
       <c r="E21" s="42" t="n">
@@ -7889,25 +7900,25 @@
         <v>113</v>
       </c>
       <c r="K21" s="58" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="L21" s="58" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="N21" s="58" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="O21" s="58" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="P21" s="48" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="Q21" s="43" t="n">
         <v>32465</v>
       </c>
       <c r="R21" s="58" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="S21" s="58" t="s">
         <v>120</v>
@@ -7915,31 +7926,31 @@
       <c r="T21" s="58"/>
       <c r="U21" s="48"/>
       <c r="V21" s="58" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="W21" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="X21" s="59" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="Y21" s="48" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="Z21" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="AA21" s="59" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="AB21" s="48" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="AC21" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="AD21" s="59" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="AE21" s="48" t="s">
         <v>147</v>
@@ -7951,7 +7962,7 @@
         <v>147</v>
       </c>
       <c r="AH21" s="63" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AI21" s="55" t="n">
         <v>45668</v>
@@ -7960,22 +7971,22 @@
         <v>0.732638888888889</v>
       </c>
       <c r="AK21" s="61" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="AL21" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM21" s="62" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="AN21" s="47" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="AO21" s="59" t="n">
         <v>45670</v>
       </c>
       <c r="AP21" s="40" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AQ21" s="40" t="s">
         <v>123</v>
@@ -8011,10 +8022,10 @@
         <v>151</v>
       </c>
       <c r="BB21" s="48" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="BC21" s="40" t="s">
-        <v>176</v>
+        <v>153</v>
       </c>
       <c r="BD21" s="42" t="n">
         <v>45671</v>
@@ -8026,7 +8037,7 @@
         <v>151</v>
       </c>
       <c r="BG21" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BH21" s="48" t="s">
         <v>147</v>
@@ -8035,19 +8046,19 @@
       <c r="BJ21" s="60"/>
       <c r="BK21" s="48"/>
       <c r="BL21" s="48" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="BM21" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN21" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BO21" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP21" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BQ21" s="42" t="n">
         <f aca="false">AL21</f>
@@ -8060,13 +8071,13 @@
         <v>135</v>
       </c>
       <c r="BT21" s="40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="BU21" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV21" s="40" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="BW21" s="42" t="n">
         <f aca="false">AO21</f>
@@ -8076,16 +8087,16 @@
         <v>18.0423611111111</v>
       </c>
       <c r="BY21" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="BZ21" s="42" t="s">
         <v>156</v>
       </c>
-      <c r="BZ21" s="42" t="s">
-        <v>154</v>
-      </c>
       <c r="CA21" s="39" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="CB21" s="39" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="CC21" s="42" t="n">
         <f aca="false">AO21</f>
@@ -29151,10 +29162,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D1" s="99" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E1" s="99" t="s">
         <v>4</v>
@@ -29163,13 +29174,13 @@
         <v>5</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="H1" s="11" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="15" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="J1" s="15" t="s">
         <v>9</v>
@@ -29184,7 +29195,7 @@
         <v>12</v>
       </c>
       <c r="N1" s="32" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="O1" s="32" t="s">
         <v>14</v>
@@ -29468,7 +29479,7 @@
         <v>115</v>
       </c>
       <c r="M2" s="32" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="N2" s="32" t="s">
         <v>117</v>
@@ -29747,25 +29758,25 @@
         <v>113</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="R3" s="2" t="s">
         <v>147</v>
@@ -29855,7 +29866,7 @@
       <c r="CN3" s="5"/>
       <c r="CO3" s="1"/>
       <c r="CQ3" s="1" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="CR3" s="1"/>
       <c r="CS3" s="1"/>

</xml_diff>

<commit_message>
- Errores avanzados (80%) (13-05-2025)
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -661,7 +661,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1479" uniqueCount="334">
   <si>
     <t xml:space="preserve">Activo</t>
   </si>
@@ -1098,6 +1098,9 @@
     <t xml:space="preserve">PANTINO</t>
   </si>
   <si>
+    <t xml:space="preserve">F</t>
+  </si>
+  <si>
     <t xml:space="preserve">Philippines</t>
   </si>
   <si>
@@ -1200,6 +1203,9 @@
     <t xml:space="preserve">Esta es una segunda prueba</t>
   </si>
   <si>
+    <t xml:space="preserve">SII</t>
+  </si>
+  <si>
     <t xml:space="preserve"> KARLA JAY</t>
   </si>
   <si>
@@ -1228,6 +1234,9 @@
   </si>
   <si>
     <t xml:space="preserve">SINGLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOO</t>
   </si>
   <si>
     <t xml:space="preserve"> BEN</t>
@@ -3318,9 +3327,11 @@
       <c r="L3" s="41" t="s">
         <v>144</v>
       </c>
-      <c r="M3" s="39"/>
+      <c r="M3" s="39" t="s">
+        <v>145</v>
+      </c>
       <c r="N3" s="41" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O3" s="41" t="s">
         <v>118</v>
@@ -3332,7 +3343,7 @@
         <v>28288</v>
       </c>
       <c r="R3" s="41" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="S3" s="41" t="s">
         <v>120</v>
@@ -3340,46 +3351,46 @@
       <c r="T3" s="41"/>
       <c r="U3" s="40"/>
       <c r="V3" s="41" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="W3" s="42"/>
       <c r="X3" s="42"/>
       <c r="Y3" s="40" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="Z3" s="42"/>
       <c r="AA3" s="42"/>
       <c r="AB3" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AC3" s="42"/>
       <c r="AD3" s="42"/>
       <c r="AE3" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF3" s="40"/>
       <c r="AG3" s="40"/>
       <c r="AH3" s="41" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AI3" s="42"/>
       <c r="AJ3" s="44"/>
       <c r="AK3" s="45" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AL3" s="42" t="n">
         <v>45660</v>
       </c>
       <c r="AM3" s="46" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="AN3" s="47" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AO3" s="42"/>
       <c r="AP3" s="46"/>
       <c r="AQ3" s="40" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="AR3" s="40" t="s">
         <v>124</v>
@@ -3398,7 +3409,7 @@
       </c>
       <c r="AW3" s="40"/>
       <c r="AX3" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY3" s="42" t="n">
         <v>45660</v>
@@ -3407,13 +3418,13 @@
         <v>45662</v>
       </c>
       <c r="BA3" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BB3" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BC3" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BD3" s="42" t="n">
         <v>45671</v>
@@ -3422,31 +3433,31 @@
         <v>45672</v>
       </c>
       <c r="BF3" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG3" s="40" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="BH3" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI3" s="43"/>
       <c r="BJ3" s="43"/>
       <c r="BK3" s="40"/>
       <c r="BL3" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BM3" s="40" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="BN3" s="40" t="s">
+        <v>157</v>
+      </c>
+      <c r="BO3" s="40" t="s">
         <v>156</v>
       </c>
-      <c r="BO3" s="40" t="s">
-        <v>155</v>
-      </c>
       <c r="BP3" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BQ3" s="42" t="n">
         <f aca="false">AL3</f>
@@ -3456,16 +3467,16 @@
         <v>0.0423611111111111</v>
       </c>
       <c r="BS3" s="40" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="BT3" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="BU3" s="40" t="s">
+        <v>156</v>
+      </c>
+      <c r="BV3" s="40" t="s">
         <v>157</v>
-      </c>
-      <c r="BU3" s="40" t="s">
-        <v>155</v>
-      </c>
-      <c r="BV3" s="40" t="s">
-        <v>156</v>
       </c>
       <c r="BW3" s="42" t="n">
         <f aca="false">AO3</f>
@@ -3475,16 +3486,16 @@
         <v>0.0423611111111111</v>
       </c>
       <c r="BY3" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BZ3" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="CA3" s="39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="CB3" s="39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="CC3" s="42" t="n">
         <f aca="false">AO3</f>
@@ -3494,7 +3505,7 @@
         <v>0.0423611111111111</v>
       </c>
       <c r="CE3" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF3" s="42"/>
       <c r="CG3" s="42"/>
@@ -3521,12 +3532,12 @@
       <c r="DA3" s="42"/>
       <c r="DB3" s="40"/>
       <c r="DC3" s="51" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4" s="51" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="39" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="B4" s="40" t="s">
         <v>108</v>
@@ -3554,26 +3565,28 @@
         <v>113</v>
       </c>
       <c r="K4" s="41" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="L4" s="41" t="s">
-        <v>162</v>
-      </c>
-      <c r="M4" s="39"/>
+        <v>163</v>
+      </c>
+      <c r="M4" s="39" t="s">
+        <v>145</v>
+      </c>
       <c r="N4" s="41" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="O4" s="41" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="P4" s="40" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="Q4" s="43" t="n">
         <v>32524</v>
       </c>
       <c r="R4" s="41" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="S4" s="41" t="s">
         <v>120</v>
@@ -3581,43 +3594,43 @@
       <c r="T4" s="41"/>
       <c r="U4" s="40"/>
       <c r="V4" s="41" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="W4" s="42" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="X4" s="42" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="Y4" s="40" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="Z4" s="42" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AA4" s="42" t="s">
+        <v>172</v>
+      </c>
+      <c r="AB4" s="40" t="s">
+        <v>173</v>
+      </c>
+      <c r="AC4" s="42" t="s">
         <v>171</v>
       </c>
-      <c r="AB4" s="40" t="s">
-        <v>172</v>
-      </c>
-      <c r="AC4" s="42" t="s">
-        <v>170</v>
-      </c>
       <c r="AD4" s="42" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="AE4" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF4" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AG4" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AH4" s="41" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="AI4" s="42" t="n">
         <v>45660</v>
@@ -3626,22 +3639,22 @@
         <v>0.40625</v>
       </c>
       <c r="AK4" s="45" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AL4" s="42" t="n">
         <v>45660</v>
       </c>
       <c r="AM4" s="46" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="AN4" s="47" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AO4" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP4" s="42" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="AQ4" s="40" t="s">
         <v>123</v>
@@ -3649,9 +3662,7 @@
       <c r="AR4" s="40" t="s">
         <v>124</v>
       </c>
-      <c r="AS4" s="40" t="s">
-        <v>125</v>
-      </c>
+      <c r="AS4" s="40"/>
       <c r="AT4" s="40" t="s">
         <v>126</v>
       </c>
@@ -3665,7 +3676,7 @@
         <v>3</v>
       </c>
       <c r="AX4" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY4" s="42" t="n">
         <v>45660</v>
@@ -3674,10 +3685,10 @@
         <v>45662</v>
       </c>
       <c r="BA4" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BB4" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BC4" s="40"/>
       <c r="BD4" s="42" t="n">
@@ -3687,31 +3698,31 @@
         <v>45672</v>
       </c>
       <c r="BF4" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG4" s="40" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="BH4" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI4" s="43"/>
       <c r="BJ4" s="43"/>
       <c r="BK4" s="40"/>
       <c r="BL4" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BM4" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN4" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BO4" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP4" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BQ4" s="42" t="n">
         <f aca="false">AL4</f>
@@ -3724,13 +3735,13 @@
         <v>135</v>
       </c>
       <c r="BT4" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BU4" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV4" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BW4" s="42" t="n">
         <f aca="false">AO4</f>
@@ -3740,16 +3751,16 @@
         <v>1.04236111111111</v>
       </c>
       <c r="BY4" s="40" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="BZ4" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="CA4" s="39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="CB4" s="39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="CC4" s="42" t="n">
         <f aca="false">AO4</f>
@@ -3759,7 +3770,7 @@
         <v>1.04236111111111</v>
       </c>
       <c r="CE4" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF4" s="42"/>
       <c r="CG4" s="42"/>
@@ -3784,12 +3795,12 @@
       <c r="DA4" s="42"/>
       <c r="DB4" s="40"/>
       <c r="DC4" s="51" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="5" s="51" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="39" t="s">
-        <v>140</v>
+        <v>180</v>
       </c>
       <c r="B5" s="40" t="s">
         <v>108</v>
@@ -3817,26 +3828,28 @@
         <v>113</v>
       </c>
       <c r="K5" s="41" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="L5" s="41" t="s">
-        <v>180</v>
-      </c>
-      <c r="M5" s="39"/>
+        <v>182</v>
+      </c>
+      <c r="M5" s="39" t="s">
+        <v>145</v>
+      </c>
       <c r="N5" s="41" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="O5" s="41" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="P5" s="40" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="Q5" s="43" t="n">
         <v>32346</v>
       </c>
       <c r="R5" s="41" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="S5" s="41" t="s">
         <v>120</v>
@@ -3844,43 +3857,43 @@
       <c r="T5" s="41"/>
       <c r="U5" s="40"/>
       <c r="V5" s="41" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="W5" s="42" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="X5" s="42" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="Y5" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="Z5" s="42" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AA5" s="42" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AB5" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AC5" s="42" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AD5" s="42" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AE5" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF5" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AG5" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AH5" s="41" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="AI5" s="42" t="n">
         <v>45661</v>
@@ -3889,22 +3902,22 @@
         <v>0.472222222222222</v>
       </c>
       <c r="AK5" s="45" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="AL5" s="42" t="n">
         <v>45661</v>
       </c>
       <c r="AM5" s="46" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="AN5" s="47" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AO5" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP5" s="40" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="AQ5" s="40" t="s">
         <v>123</v>
@@ -3918,9 +3931,7 @@
       <c r="AT5" s="40" t="s">
         <v>126</v>
       </c>
-      <c r="AU5" s="40" t="s">
-        <v>127</v>
-      </c>
+      <c r="AU5" s="40"/>
       <c r="AV5" s="40" t="s">
         <v>128</v>
       </c>
@@ -3928,7 +3939,7 @@
         <v>3</v>
       </c>
       <c r="AX5" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY5" s="42" t="n">
         <v>45661</v>
@@ -3937,13 +3948,13 @@
         <v>45662</v>
       </c>
       <c r="BA5" s="40" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="BB5" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BC5" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BD5" s="42" t="n">
         <v>45671</v>
@@ -3952,31 +3963,31 @@
         <v>45672</v>
       </c>
       <c r="BF5" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG5" s="40" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="BH5" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI5" s="43"/>
       <c r="BJ5" s="43"/>
       <c r="BK5" s="40"/>
       <c r="BL5" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BM5" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN5" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BO5" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP5" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BQ5" s="42" t="n">
         <f aca="false">AL5</f>
@@ -3989,13 +4000,13 @@
         <v>135</v>
       </c>
       <c r="BT5" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BU5" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV5" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BW5" s="42" t="n">
         <f aca="false">AO5</f>
@@ -4005,16 +4016,16 @@
         <v>2.04236111111111</v>
       </c>
       <c r="BY5" s="40" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="BZ5" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="CA5" s="39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="CB5" s="39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="CC5" s="42" t="n">
         <f aca="false">AO5</f>
@@ -4024,7 +4035,7 @@
         <v>2.04236111111111</v>
       </c>
       <c r="CE5" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF5" s="42"/>
       <c r="CG5" s="42"/>
@@ -4053,7 +4064,7 @@
     </row>
     <row r="6" s="51" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="39" t="s">
-        <v>140</v>
+        <v>191</v>
       </c>
       <c r="B6" s="40" t="s">
         <v>108</v>
@@ -4081,20 +4092,22 @@
         <v>113</v>
       </c>
       <c r="K6" s="41" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="L6" s="41" t="s">
-        <v>190</v>
-      </c>
-      <c r="M6" s="39"/>
+        <v>193</v>
+      </c>
+      <c r="M6" s="39" t="s">
+        <v>145</v>
+      </c>
       <c r="N6" s="41" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="O6" s="41" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="P6" s="40" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="Q6" s="43" t="n">
         <v>30193</v>
@@ -4106,43 +4119,43 @@
       <c r="T6" s="41"/>
       <c r="U6" s="40"/>
       <c r="V6" s="41" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="W6" s="42" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="X6" s="42" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="Y6" s="40" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="Z6" s="42" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AA6" s="42" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="AB6" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AC6" s="42" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AD6" s="42" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AE6" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF6" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AG6" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AH6" s="41" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="AI6" s="42" t="n">
         <v>45661</v>
@@ -4151,22 +4164,22 @@
         <v>0.388888888888889</v>
       </c>
       <c r="AK6" s="45" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="AL6" s="42" t="n">
         <v>45661</v>
       </c>
       <c r="AM6" s="46" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="AN6" s="47" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AO6" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP6" s="40" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="AQ6" s="40" t="s">
         <v>123</v>
@@ -4190,7 +4203,7 @@
         <v>3</v>
       </c>
       <c r="AX6" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY6" s="42" t="n">
         <v>45661</v>
@@ -4199,13 +4212,13 @@
         <v>45662</v>
       </c>
       <c r="BA6" s="40" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="BB6" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BC6" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BD6" s="42" t="n">
         <v>45671</v>
@@ -4214,31 +4227,31 @@
         <v>45672</v>
       </c>
       <c r="BF6" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG6" s="40" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="BH6" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI6" s="43"/>
       <c r="BJ6" s="43"/>
       <c r="BK6" s="40"/>
       <c r="BL6" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BM6" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN6" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BO6" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP6" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BQ6" s="42" t="n">
         <f aca="false">AL6</f>
@@ -4251,13 +4264,13 @@
         <v>135</v>
       </c>
       <c r="BT6" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BU6" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV6" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BW6" s="42" t="n">
         <f aca="false">AO6</f>
@@ -4267,16 +4280,16 @@
         <v>3.04236111111111</v>
       </c>
       <c r="BY6" s="40" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="BZ6" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="CA6" s="39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="CB6" s="39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="CC6" s="42" t="n">
         <f aca="false">AO6</f>
@@ -4286,7 +4299,7 @@
         <v>3.04236111111111</v>
       </c>
       <c r="CE6" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF6" s="42"/>
       <c r="CG6" s="42"/>
@@ -4312,9 +4325,7 @@
       <c r="DB6" s="40"/>
     </row>
     <row r="7" s="51" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="39" t="s">
-        <v>140</v>
-      </c>
+      <c r="A7" s="39"/>
       <c r="B7" s="40" t="s">
         <v>108</v>
       </c>
@@ -4341,72 +4352,74 @@
         <v>113</v>
       </c>
       <c r="K7" s="41" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="L7" s="41" t="s">
-        <v>200</v>
-      </c>
-      <c r="M7" s="39"/>
+        <v>203</v>
+      </c>
+      <c r="M7" s="39" t="s">
+        <v>145</v>
+      </c>
       <c r="N7" s="41" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="O7" s="41" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="P7" s="40" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="Q7" s="43" t="n">
         <v>36383</v>
       </c>
       <c r="R7" s="41" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="S7" s="41" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="T7" s="41" t="s">
         <v>120</v>
       </c>
       <c r="U7" s="40"/>
       <c r="V7" s="41" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="W7" s="42" t="n">
         <v>45661</v>
       </c>
       <c r="X7" s="42" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="Y7" s="40" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="Z7" s="42" t="n">
         <v>45661</v>
       </c>
       <c r="AA7" s="42" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="AB7" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AC7" s="42" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AD7" s="42" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AE7" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF7" s="43" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AG7" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AH7" s="41" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="AI7" s="42" t="n">
         <v>45661</v>
@@ -4415,22 +4428,22 @@
         <v>0.451388888888889</v>
       </c>
       <c r="AK7" s="45" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="AL7" s="42" t="n">
         <v>45661</v>
       </c>
       <c r="AM7" s="46" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="AN7" s="47" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AO7" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP7" s="40" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="AQ7" s="40" t="s">
         <v>123</v>
@@ -4454,7 +4467,7 @@
         <v>3</v>
       </c>
       <c r="AX7" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY7" s="42" t="n">
         <v>45661</v>
@@ -4463,13 +4476,13 @@
         <v>45662</v>
       </c>
       <c r="BA7" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BB7" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BC7" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BD7" s="42" t="n">
         <v>45671</v>
@@ -4478,31 +4491,31 @@
         <v>45672</v>
       </c>
       <c r="BF7" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG7" s="40" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="BH7" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI7" s="43"/>
       <c r="BJ7" s="43"/>
       <c r="BK7" s="40"/>
       <c r="BL7" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BM7" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN7" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BO7" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP7" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BQ7" s="42" t="n">
         <f aca="false">AL7</f>
@@ -4515,13 +4528,13 @@
         <v>135</v>
       </c>
       <c r="BT7" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BU7" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV7" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BW7" s="42" t="n">
         <f aca="false">AO7</f>
@@ -4531,16 +4544,16 @@
         <v>4.04236111111111</v>
       </c>
       <c r="BY7" s="40" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="BZ7" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="CA7" s="39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="CB7" s="39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="CC7" s="42" t="n">
         <f aca="false">AO7</f>
@@ -4550,7 +4563,7 @@
         <v>4.04236111111111</v>
       </c>
       <c r="CE7" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF7" s="42"/>
       <c r="CG7" s="42"/>
@@ -4607,26 +4620,28 @@
         <v>113</v>
       </c>
       <c r="K8" s="41" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="L8" s="41" t="s">
-        <v>211</v>
-      </c>
-      <c r="M8" s="39"/>
+        <v>214</v>
+      </c>
+      <c r="M8" s="39" t="s">
+        <v>145</v>
+      </c>
       <c r="N8" s="41" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="O8" s="41" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="P8" s="40" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="Q8" s="43" t="n">
         <v>29208</v>
       </c>
       <c r="R8" s="41" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="S8" s="41" t="s">
         <v>120</v>
@@ -4634,43 +4649,43 @@
       <c r="T8" s="41"/>
       <c r="U8" s="40"/>
       <c r="V8" s="52" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="W8" s="53" t="n">
         <v>45667</v>
       </c>
       <c r="X8" s="53" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="Y8" s="54" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="Z8" s="53" t="n">
         <v>45668</v>
       </c>
       <c r="AA8" s="53" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="AB8" s="54" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="AC8" s="53" t="n">
         <v>45668</v>
       </c>
       <c r="AD8" s="53" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="AE8" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF8" s="43" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AG8" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AH8" s="41" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="AI8" s="42" t="n">
         <v>45661</v>
@@ -4679,22 +4694,22 @@
         <v>0.451388888888889</v>
       </c>
       <c r="AK8" s="45" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="AL8" s="42" t="n">
         <v>45661</v>
       </c>
       <c r="AM8" s="46" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="AN8" s="47" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AO8" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP8" s="40" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="AQ8" s="40" t="s">
         <v>123</v>
@@ -4718,7 +4733,7 @@
         <v>1</v>
       </c>
       <c r="AX8" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY8" s="42" t="n">
         <v>45661</v>
@@ -4727,13 +4742,13 @@
         <v>45662</v>
       </c>
       <c r="BA8" s="40" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="BB8" s="40" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="BC8" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BD8" s="42" t="n">
         <v>45671</v>
@@ -4742,31 +4757,31 @@
         <v>45672</v>
       </c>
       <c r="BF8" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG8" s="40" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="BH8" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI8" s="43"/>
       <c r="BJ8" s="43"/>
       <c r="BK8" s="40"/>
       <c r="BL8" s="40" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="BM8" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN8" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BO8" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP8" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BQ8" s="42" t="n">
         <f aca="false">AL8</f>
@@ -4779,13 +4794,13 @@
         <v>135</v>
       </c>
       <c r="BT8" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BU8" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV8" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BW8" s="42" t="n">
         <f aca="false">AO8</f>
@@ -4795,16 +4810,16 @@
         <v>5.04236111111111</v>
       </c>
       <c r="BY8" s="40" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="BZ8" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="CA8" s="39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="CB8" s="39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="CC8" s="42" t="n">
         <f aca="false">AO8</f>
@@ -4814,7 +4829,7 @@
         <v>5.04236111111111</v>
       </c>
       <c r="CE8" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF8" s="42"/>
       <c r="CG8" s="42"/>
@@ -4864,26 +4879,28 @@
         <v>113</v>
       </c>
       <c r="K9" s="41" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="L9" s="41" t="s">
-        <v>223</v>
-      </c>
-      <c r="M9" s="39"/>
+        <v>226</v>
+      </c>
+      <c r="M9" s="39" t="s">
+        <v>145</v>
+      </c>
       <c r="N9" s="41" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="O9" s="41" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="P9" s="40" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="Q9" s="43" t="n">
         <v>33062</v>
       </c>
       <c r="R9" s="41" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="S9" s="41" t="s">
         <v>120</v>
@@ -4891,43 +4908,43 @@
       <c r="T9" s="41"/>
       <c r="U9" s="40"/>
       <c r="V9" s="41" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="W9" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X9" s="42" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="Y9" s="40" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="Z9" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA9" s="42" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="AB9" s="40" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="AC9" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AD9" s="42" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="AE9" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF9" s="43" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AG9" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AH9" s="41" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="AI9" s="42" t="n">
         <v>45661</v>
@@ -4936,22 +4953,22 @@
         <v>0.409722222222222</v>
       </c>
       <c r="AK9" s="45" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="AL9" s="42" t="n">
         <v>45661</v>
       </c>
       <c r="AM9" s="46" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="AN9" s="47" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AO9" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP9" s="40" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="AQ9" s="40" t="s">
         <v>123</v>
@@ -4975,7 +4992,7 @@
         <v>3</v>
       </c>
       <c r="AX9" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY9" s="42" t="n">
         <v>45661</v>
@@ -4984,13 +5001,13 @@
         <v>45662</v>
       </c>
       <c r="BA9" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BB9" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BC9" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BD9" s="42" t="n">
         <v>45671</v>
@@ -4999,31 +5016,31 @@
         <v>45672</v>
       </c>
       <c r="BF9" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG9" s="40" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="BH9" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI9" s="43"/>
       <c r="BJ9" s="43"/>
       <c r="BK9" s="40"/>
       <c r="BL9" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BM9" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN9" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BO9" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP9" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BQ9" s="42" t="n">
         <f aca="false">AL9</f>
@@ -5036,13 +5053,13 @@
         <v>135</v>
       </c>
       <c r="BT9" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BU9" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV9" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BW9" s="42" t="n">
         <f aca="false">AO9</f>
@@ -5052,16 +5069,16 @@
         <v>6.04236111111111</v>
       </c>
       <c r="BY9" s="40" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="BZ9" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="CA9" s="39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="CB9" s="39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="CC9" s="42" t="n">
         <f aca="false">AO9</f>
@@ -5071,7 +5088,7 @@
         <v>6.04236111111111</v>
       </c>
       <c r="CE9" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF9" s="42"/>
       <c r="CG9" s="42"/>
@@ -5099,7 +5116,7 @@
         <v>108</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="D10" s="42"/>
       <c r="E10" s="42" t="n">
@@ -5109,7 +5126,7 @@
         <v>45663</v>
       </c>
       <c r="G10" s="40" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="H10" s="40" t="s">
         <v>142</v>
@@ -5121,26 +5138,28 @@
         <v>113</v>
       </c>
       <c r="K10" s="41" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="L10" s="41" t="s">
-        <v>232</v>
-      </c>
-      <c r="M10" s="39"/>
+        <v>235</v>
+      </c>
+      <c r="M10" s="39" t="s">
+        <v>145</v>
+      </c>
       <c r="N10" s="41" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="O10" s="41" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="P10" s="40" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="Q10" s="43" t="n">
         <v>33794</v>
       </c>
       <c r="R10" s="41" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="S10" s="41" t="s">
         <v>120</v>
@@ -5148,43 +5167,43 @@
       <c r="T10" s="41"/>
       <c r="U10" s="40"/>
       <c r="V10" s="41" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="W10" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X10" s="42" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="Y10" s="40" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="Z10" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA10" s="42" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="AB10" s="40" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="AC10" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AD10" s="42" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="AE10" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF10" s="43" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AG10" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AH10" s="41" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="AI10" s="42" t="n">
         <v>45662</v>
@@ -5193,16 +5212,16 @@
         <v>0.40625</v>
       </c>
       <c r="AK10" s="45" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="AL10" s="42" t="n">
         <v>45662</v>
       </c>
       <c r="AM10" s="46" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="AN10" s="47" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AO10" s="42"/>
       <c r="AP10" s="40"/>
@@ -5228,7 +5247,7 @@
         <v>3</v>
       </c>
       <c r="AX10" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY10" s="42" t="n">
         <v>45662</v>
@@ -5237,13 +5256,13 @@
         <v>45663</v>
       </c>
       <c r="BA10" s="40" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="BB10" s="40" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="BC10" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BD10" s="42" t="n">
         <v>45671</v>
@@ -5252,31 +5271,31 @@
         <v>45672</v>
       </c>
       <c r="BF10" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG10" s="40" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="BH10" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI10" s="43"/>
       <c r="BJ10" s="43"/>
       <c r="BK10" s="40"/>
       <c r="BL10" s="40" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="BM10" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN10" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BO10" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP10" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BQ10" s="42" t="n">
         <f aca="false">AL10</f>
@@ -5289,13 +5308,13 @@
         <v>135</v>
       </c>
       <c r="BT10" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BU10" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV10" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BW10" s="42" t="n">
         <f aca="false">AO10</f>
@@ -5305,16 +5324,16 @@
         <v>7.04236111111111</v>
       </c>
       <c r="BY10" s="40" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="BZ10" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="CA10" s="39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="CB10" s="39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="CC10" s="55" t="n">
         <v>36892</v>
@@ -5323,7 +5342,7 @@
         <v>7.04236111111111</v>
       </c>
       <c r="CE10" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF10" s="42"/>
       <c r="CG10" s="42"/>
@@ -5373,26 +5392,28 @@
         <v>113</v>
       </c>
       <c r="K11" s="41" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="L11" s="41" t="s">
-        <v>240</v>
-      </c>
-      <c r="M11" s="39"/>
+        <v>243</v>
+      </c>
+      <c r="M11" s="39" t="s">
+        <v>145</v>
+      </c>
       <c r="N11" s="41" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="O11" s="41" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="P11" s="40" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="Q11" s="43" t="n">
         <v>33386</v>
       </c>
       <c r="R11" s="41" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="S11" s="41" t="s">
         <v>120</v>
@@ -5400,43 +5421,43 @@
       <c r="T11" s="41"/>
       <c r="U11" s="40"/>
       <c r="V11" s="41" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="W11" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X11" s="42" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="Y11" s="40" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="Z11" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA11" s="42" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="AB11" s="40" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="AC11" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AD11" s="42" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="AE11" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF11" s="43" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AG11" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AH11" s="41" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AI11" s="42" t="n">
         <v>45665</v>
@@ -5445,22 +5466,22 @@
         <v>0.354166666666667</v>
       </c>
       <c r="AK11" s="45" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AL11" s="42" t="n">
         <v>45665</v>
       </c>
       <c r="AM11" s="46" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AN11" s="57" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="AO11" s="42" t="n">
         <v>45665</v>
       </c>
       <c r="AP11" s="40" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="AQ11" s="40" t="s">
         <v>123</v>
@@ -5484,7 +5505,7 @@
         <v>1</v>
       </c>
       <c r="AX11" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY11" s="42" t="n">
         <v>45662</v>
@@ -5493,13 +5514,13 @@
         <v>45663</v>
       </c>
       <c r="BA11" s="40" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="BB11" s="40" t="s">
+        <v>155</v>
+      </c>
+      <c r="BC11" s="40" t="s">
         <v>154</v>
-      </c>
-      <c r="BC11" s="40" t="s">
-        <v>153</v>
       </c>
       <c r="BD11" s="42" t="n">
         <v>45671</v>
@@ -5508,22 +5529,22 @@
         <v>45672</v>
       </c>
       <c r="BF11" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG11" s="40" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="BH11" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI11" s="43"/>
       <c r="BJ11" s="43"/>
       <c r="BK11" s="40"/>
       <c r="BL11" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BM11" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BN11" s="40"/>
       <c r="BO11" s="40"/>
@@ -5531,7 +5552,7 @@
       <c r="BQ11" s="42"/>
       <c r="BR11" s="44"/>
       <c r="BS11" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BT11" s="40"/>
       <c r="BU11" s="40"/>
@@ -5539,7 +5560,7 @@
       <c r="BW11" s="42"/>
       <c r="BX11" s="44"/>
       <c r="BY11" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BZ11" s="42"/>
       <c r="CA11" s="39"/>
@@ -5547,7 +5568,7 @@
       <c r="CC11" s="42"/>
       <c r="CD11" s="44"/>
       <c r="CE11" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF11" s="42"/>
       <c r="CG11" s="42"/>
@@ -5575,7 +5596,7 @@
         <v>108</v>
       </c>
       <c r="C12" s="41" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="D12" s="42"/>
       <c r="E12" s="42" t="n">
@@ -5597,70 +5618,72 @@
         <v>113</v>
       </c>
       <c r="K12" s="41" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="L12" s="41" t="s">
-        <v>254</v>
-      </c>
-      <c r="M12" s="39"/>
+        <v>257</v>
+      </c>
+      <c r="M12" s="39" t="s">
+        <v>145</v>
+      </c>
       <c r="N12" s="41" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O12" s="41" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="P12" s="40" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="Q12" s="43" t="n">
         <v>35988</v>
       </c>
       <c r="R12" s="41" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="S12" s="41" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="T12" s="41"/>
       <c r="U12" s="40"/>
       <c r="V12" s="41" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="W12" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X12" s="42" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="Y12" s="40" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="Z12" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA12" s="42" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="AB12" s="40" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="AC12" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AD12" s="42" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="AE12" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF12" s="43" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AG12" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AH12" s="41" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="AI12" s="42" t="n">
         <v>45668</v>
@@ -5669,22 +5692,22 @@
         <v>0.732638888888889</v>
       </c>
       <c r="AK12" s="45" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="AL12" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM12" s="46" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="AN12" s="47" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="AO12" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP12" s="40" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="AQ12" s="40" t="s">
         <v>123</v>
@@ -5708,7 +5731,7 @@
         <v>3</v>
       </c>
       <c r="AX12" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY12" s="42" t="n">
         <v>45668</v>
@@ -5717,13 +5740,13 @@
         <v>45670</v>
       </c>
       <c r="BA12" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BB12" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BC12" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BD12" s="42" t="n">
         <v>45671</v>
@@ -5732,31 +5755,31 @@
         <v>45672</v>
       </c>
       <c r="BF12" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG12" s="40" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="BH12" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI12" s="43"/>
       <c r="BJ12" s="43"/>
       <c r="BK12" s="40"/>
       <c r="BL12" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BM12" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN12" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BO12" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP12" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BQ12" s="42" t="n">
         <f aca="false">AL12</f>
@@ -5769,13 +5792,13 @@
         <v>135</v>
       </c>
       <c r="BT12" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BU12" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV12" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BW12" s="42" t="n">
         <f aca="false">AO12</f>
@@ -5785,16 +5808,16 @@
         <v>9.04236111111111</v>
       </c>
       <c r="BY12" s="40" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="BZ12" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="CA12" s="39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="CB12" s="39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="CC12" s="42" t="n">
         <f aca="false">AO12</f>
@@ -5804,7 +5827,7 @@
         <v>9.04236111111111</v>
       </c>
       <c r="CE12" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF12" s="42"/>
       <c r="CG12" s="42"/>
@@ -5832,7 +5855,7 @@
         <v>108</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="D13" s="42"/>
       <c r="E13" s="42" t="n">
@@ -5854,26 +5877,28 @@
         <v>113</v>
       </c>
       <c r="K13" s="41" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="L13" s="41" t="s">
-        <v>264</v>
-      </c>
-      <c r="M13" s="39"/>
+        <v>267</v>
+      </c>
+      <c r="M13" s="39" t="s">
+        <v>145</v>
+      </c>
       <c r="N13" s="41" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O13" s="41" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="P13" s="40" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="Q13" s="43" t="n">
         <v>29371</v>
       </c>
       <c r="R13" s="41" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="S13" s="41" t="s">
         <v>120</v>
@@ -5881,43 +5906,43 @@
       <c r="T13" s="41"/>
       <c r="U13" s="40"/>
       <c r="V13" s="41" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="W13" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X13" s="42" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="Y13" s="40" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="Z13" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA13" s="42" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="AB13" s="40" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="AC13" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AD13" s="42" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="AE13" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF13" s="43" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AG13" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AH13" s="41" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="AI13" s="42" t="n">
         <v>45668</v>
@@ -5926,22 +5951,22 @@
         <v>0.732638888888889</v>
       </c>
       <c r="AK13" s="45" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="AL13" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM13" s="46" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="AN13" s="47" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="AO13" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP13" s="40" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="AQ13" s="40" t="s">
         <v>123</v>
@@ -5965,7 +5990,7 @@
         <v>3</v>
       </c>
       <c r="AX13" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY13" s="42" t="n">
         <v>45668</v>
@@ -5974,13 +5999,13 @@
         <v>45670</v>
       </c>
       <c r="BA13" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BB13" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BC13" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BD13" s="42" t="n">
         <v>45671</v>
@@ -5989,31 +6014,31 @@
         <v>45672</v>
       </c>
       <c r="BF13" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG13" s="40" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="BH13" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI13" s="43"/>
       <c r="BJ13" s="43"/>
       <c r="BK13" s="40"/>
       <c r="BL13" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BM13" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN13" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BO13" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP13" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BQ13" s="42" t="n">
         <f aca="false">AL13</f>
@@ -6026,13 +6051,13 @@
         <v>135</v>
       </c>
       <c r="BT13" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BU13" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV13" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BW13" s="42" t="n">
         <f aca="false">AO13</f>
@@ -6042,16 +6067,16 @@
         <v>10.0423611111111</v>
       </c>
       <c r="BY13" s="40" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="BZ13" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="CA13" s="39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="CB13" s="39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="CC13" s="42" t="n">
         <f aca="false">AO13</f>
@@ -6061,7 +6086,7 @@
         <v>10.0423611111111</v>
       </c>
       <c r="CE13" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF13" s="42"/>
       <c r="CG13" s="42"/>
@@ -6089,7 +6114,7 @@
         <v>108</v>
       </c>
       <c r="C14" s="41" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="D14" s="42"/>
       <c r="E14" s="42" t="n">
@@ -6111,26 +6136,28 @@
         <v>113</v>
       </c>
       <c r="K14" s="41" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="L14" s="41" t="s">
-        <v>270</v>
-      </c>
-      <c r="M14" s="39"/>
+        <v>273</v>
+      </c>
+      <c r="M14" s="39" t="s">
+        <v>145</v>
+      </c>
       <c r="N14" s="41" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O14" s="41" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="P14" s="40" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="Q14" s="43" t="n">
         <v>32894</v>
       </c>
       <c r="R14" s="41" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="S14" s="41" t="s">
         <v>120</v>
@@ -6138,43 +6165,43 @@
       <c r="T14" s="41"/>
       <c r="U14" s="40"/>
       <c r="V14" s="41" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="W14" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X14" s="42" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="Y14" s="40" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="Z14" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA14" s="42" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="AB14" s="40" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="AC14" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AD14" s="42" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="AE14" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF14" s="43" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AG14" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AH14" s="41" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="AI14" s="42" t="n">
         <v>45668</v>
@@ -6183,22 +6210,22 @@
         <v>0.590277777777778</v>
       </c>
       <c r="AK14" s="45" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="AL14" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM14" s="46" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="AN14" s="47" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="AO14" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP14" s="40" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="AQ14" s="40" t="s">
         <v>123</v>
@@ -6222,7 +6249,7 @@
         <v>3</v>
       </c>
       <c r="AX14" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY14" s="42" t="n">
         <v>45668</v>
@@ -6231,13 +6258,13 @@
         <v>45670</v>
       </c>
       <c r="BA14" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BB14" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BC14" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BD14" s="42" t="n">
         <v>45671</v>
@@ -6246,31 +6273,31 @@
         <v>45672</v>
       </c>
       <c r="BF14" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG14" s="40" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="BH14" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI14" s="43"/>
       <c r="BJ14" s="43"/>
       <c r="BK14" s="40"/>
       <c r="BL14" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BM14" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN14" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BO14" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP14" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BQ14" s="42" t="n">
         <f aca="false">AL14</f>
@@ -6283,13 +6310,13 @@
         <v>135</v>
       </c>
       <c r="BT14" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BU14" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV14" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BW14" s="42" t="n">
         <f aca="false">AO14</f>
@@ -6299,16 +6326,16 @@
         <v>11.0423611111111</v>
       </c>
       <c r="BY14" s="40" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="BZ14" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="CA14" s="39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="CB14" s="39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="CC14" s="42" t="n">
         <f aca="false">AO14</f>
@@ -6318,7 +6345,7 @@
         <v>11.0423611111111</v>
       </c>
       <c r="CE14" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF14" s="42"/>
       <c r="CG14" s="42"/>
@@ -6346,7 +6373,7 @@
         <v>108</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="D15" s="42"/>
       <c r="E15" s="42" t="n">
@@ -6368,26 +6395,28 @@
         <v>113</v>
       </c>
       <c r="K15" s="41" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="L15" s="41" t="s">
-        <v>276</v>
-      </c>
-      <c r="M15" s="39"/>
+        <v>279</v>
+      </c>
+      <c r="M15" s="39" t="s">
+        <v>145</v>
+      </c>
       <c r="N15" s="41" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O15" s="41" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="P15" s="40" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="Q15" s="43" t="n">
         <v>32113</v>
       </c>
       <c r="R15" s="41" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="S15" s="41" t="s">
         <v>120</v>
@@ -6395,43 +6424,43 @@
       <c r="T15" s="41"/>
       <c r="U15" s="40"/>
       <c r="V15" s="41" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="W15" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X15" s="42" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="Y15" s="40" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="Z15" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA15" s="42" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="AB15" s="40" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="AC15" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AD15" s="42" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="AE15" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF15" s="43" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AG15" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AH15" s="41" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="AI15" s="42" t="n">
         <v>45668</v>
@@ -6440,22 +6469,22 @@
         <v>0.590277777777778</v>
       </c>
       <c r="AK15" s="45" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="AL15" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM15" s="46" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="AN15" s="47" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="AO15" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP15" s="40" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="AQ15" s="40" t="s">
         <v>123</v>
@@ -6479,7 +6508,7 @@
         <v>3</v>
       </c>
       <c r="AX15" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY15" s="42" t="n">
         <v>45668</v>
@@ -6488,13 +6517,13 @@
         <v>45670</v>
       </c>
       <c r="BA15" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BB15" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BC15" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BD15" s="42" t="n">
         <v>45671</v>
@@ -6503,31 +6532,31 @@
         <v>45672</v>
       </c>
       <c r="BF15" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG15" s="40" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="BH15" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI15" s="43"/>
       <c r="BJ15" s="43"/>
       <c r="BK15" s="40"/>
       <c r="BL15" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BM15" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN15" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BO15" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP15" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BQ15" s="42" t="n">
         <f aca="false">AL15</f>
@@ -6540,13 +6569,13 @@
         <v>135</v>
       </c>
       <c r="BT15" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BU15" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV15" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BW15" s="42" t="n">
         <f aca="false">AO15</f>
@@ -6556,16 +6585,16 @@
         <v>12.0423611111111</v>
       </c>
       <c r="BY15" s="40" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="BZ15" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="CA15" s="39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="CB15" s="39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="CC15" s="42" t="n">
         <f aca="false">AO15</f>
@@ -6575,7 +6604,7 @@
         <v>12.0423611111111</v>
       </c>
       <c r="CE15" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF15" s="42"/>
       <c r="CG15" s="42"/>
@@ -6603,7 +6632,7 @@
         <v>108</v>
       </c>
       <c r="C16" s="41" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="D16" s="42"/>
       <c r="E16" s="42" t="n">
@@ -6625,70 +6654,72 @@
         <v>113</v>
       </c>
       <c r="K16" s="41" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="L16" s="41" t="s">
-        <v>280</v>
-      </c>
-      <c r="M16" s="39"/>
+        <v>283</v>
+      </c>
+      <c r="M16" s="39" t="s">
+        <v>145</v>
+      </c>
       <c r="N16" s="41" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O16" s="41" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="P16" s="40" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="Q16" s="43" t="n">
         <v>35754</v>
       </c>
       <c r="R16" s="41" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="S16" s="41" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="T16" s="41"/>
       <c r="U16" s="40"/>
       <c r="V16" s="41" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="W16" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X16" s="42" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="Y16" s="40" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="Z16" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA16" s="42" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="AB16" s="40" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="AC16" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AD16" s="42" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="AE16" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF16" s="43" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AG16" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AH16" s="41" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="AI16" s="42" t="n">
         <v>45668</v>
@@ -6697,22 +6728,22 @@
         <v>0.732638888888889</v>
       </c>
       <c r="AK16" s="45" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="AL16" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM16" s="46" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="AN16" s="47" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="AO16" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP16" s="40" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="AQ16" s="40" t="s">
         <v>123</v>
@@ -6736,7 +6767,7 @@
         <v>3</v>
       </c>
       <c r="AX16" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY16" s="42" t="n">
         <v>45668</v>
@@ -6745,13 +6776,13 @@
         <v>45670</v>
       </c>
       <c r="BA16" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BB16" s="40" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="BC16" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BD16" s="42" t="n">
         <v>45671</v>
@@ -6760,31 +6791,31 @@
         <v>45672</v>
       </c>
       <c r="BF16" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG16" s="40" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="BH16" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI16" s="43"/>
       <c r="BJ16" s="43"/>
       <c r="BK16" s="40"/>
       <c r="BL16" s="40" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="BM16" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN16" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BO16" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP16" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BQ16" s="42" t="n">
         <f aca="false">AL16</f>
@@ -6797,13 +6828,13 @@
         <v>135</v>
       </c>
       <c r="BT16" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BU16" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV16" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BW16" s="42" t="n">
         <f aca="false">AO16</f>
@@ -6813,16 +6844,16 @@
         <v>13.0423611111111</v>
       </c>
       <c r="BY16" s="40" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="BZ16" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="CA16" s="39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="CB16" s="39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="CC16" s="42" t="n">
         <f aca="false">AO16</f>
@@ -6832,7 +6863,7 @@
         <v>13.0423611111111</v>
       </c>
       <c r="CE16" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF16" s="42"/>
       <c r="CG16" s="42"/>
@@ -6860,7 +6891,7 @@
         <v>108</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="D17" s="42"/>
       <c r="E17" s="42" t="n">
@@ -6882,26 +6913,28 @@
         <v>113</v>
       </c>
       <c r="K17" s="41" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="L17" s="41" t="s">
-        <v>285</v>
-      </c>
-      <c r="M17" s="39"/>
+        <v>288</v>
+      </c>
+      <c r="M17" s="39" t="s">
+        <v>145</v>
+      </c>
       <c r="N17" s="41" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O17" s="41" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="P17" s="40" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="Q17" s="43" t="n">
         <v>33264</v>
       </c>
       <c r="R17" s="41" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="S17" s="41" t="s">
         <v>120</v>
@@ -6909,43 +6942,43 @@
       <c r="T17" s="41"/>
       <c r="U17" s="40"/>
       <c r="V17" s="41" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="W17" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X17" s="42" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="Y17" s="40" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="Z17" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA17" s="42" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="AB17" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AC17" s="42" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AD17" s="42" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AE17" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF17" s="43" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AG17" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AH17" s="41" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="AI17" s="42" t="n">
         <v>45668</v>
@@ -6954,22 +6987,22 @@
         <v>0.590277777777778</v>
       </c>
       <c r="AK17" s="45" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="AL17" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM17" s="46" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="AN17" s="47" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="AO17" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP17" s="40" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="AQ17" s="40" t="s">
         <v>123</v>
@@ -6993,7 +7026,7 @@
         <v>3</v>
       </c>
       <c r="AX17" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY17" s="42" t="n">
         <v>45668</v>
@@ -7002,13 +7035,13 @@
         <v>45670</v>
       </c>
       <c r="BA17" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BB17" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BC17" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BD17" s="42" t="n">
         <v>45671</v>
@@ -7017,31 +7050,31 @@
         <v>45672</v>
       </c>
       <c r="BF17" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG17" s="40" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="BH17" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI17" s="43"/>
       <c r="BJ17" s="43"/>
       <c r="BK17" s="40"/>
       <c r="BL17" s="40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BM17" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN17" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BO17" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP17" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BQ17" s="42" t="n">
         <f aca="false">AL17</f>
@@ -7054,13 +7087,13 @@
         <v>135</v>
       </c>
       <c r="BT17" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BU17" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV17" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BW17" s="42" t="n">
         <f aca="false">AO17</f>
@@ -7070,16 +7103,16 @@
         <v>14.0423611111111</v>
       </c>
       <c r="BY17" s="40" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="BZ17" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="CA17" s="39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="CB17" s="39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="CC17" s="42" t="n">
         <f aca="false">AO17</f>
@@ -7089,7 +7122,7 @@
         <v>14.0423611111111</v>
       </c>
       <c r="CE17" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF17" s="42"/>
       <c r="CG17" s="42"/>
@@ -7117,7 +7150,7 @@
         <v>108</v>
       </c>
       <c r="C18" s="41" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="D18" s="42"/>
       <c r="E18" s="42" t="n">
@@ -7139,70 +7172,72 @@
         <v>113</v>
       </c>
       <c r="K18" s="41" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="L18" s="41" t="s">
-        <v>292</v>
-      </c>
-      <c r="M18" s="39"/>
+        <v>295</v>
+      </c>
+      <c r="M18" s="39" t="s">
+        <v>145</v>
+      </c>
       <c r="N18" s="41" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O18" s="41" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="P18" s="40" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="Q18" s="43" t="n">
         <v>28156</v>
       </c>
       <c r="R18" s="41" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="S18" s="41" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="T18" s="41"/>
       <c r="U18" s="40"/>
       <c r="V18" s="41" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="W18" s="42" t="n">
         <v>45667</v>
       </c>
       <c r="X18" s="42" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="Y18" s="40" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="Z18" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AA18" s="42" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="AB18" s="40" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="AC18" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AD18" s="42" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="AE18" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF18" s="43" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AG18" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AH18" s="41" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="AI18" s="42" t="n">
         <v>45668</v>
@@ -7211,22 +7246,22 @@
         <v>0.732638888888889</v>
       </c>
       <c r="AK18" s="45" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="AL18" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM18" s="46" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="AN18" s="47" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="AO18" s="42" t="n">
         <v>45670</v>
       </c>
       <c r="AP18" s="40" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="AQ18" s="40" t="s">
         <v>123</v>
@@ -7250,7 +7285,7 @@
         <v>3</v>
       </c>
       <c r="AX18" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY18" s="42" t="n">
         <v>45668</v>
@@ -7259,13 +7294,13 @@
         <v>45670</v>
       </c>
       <c r="BA18" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BB18" s="40" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="BC18" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BD18" s="42" t="n">
         <v>45671</v>
@@ -7274,31 +7309,31 @@
         <v>45672</v>
       </c>
       <c r="BF18" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG18" s="40" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="BH18" s="40" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI18" s="43"/>
       <c r="BJ18" s="43"/>
       <c r="BK18" s="40"/>
       <c r="BL18" s="40" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="BM18" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN18" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BO18" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP18" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BQ18" s="42" t="n">
         <f aca="false">AL18</f>
@@ -7311,13 +7346,13 @@
         <v>135</v>
       </c>
       <c r="BT18" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BU18" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV18" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BW18" s="42" t="n">
         <f aca="false">AO18</f>
@@ -7327,16 +7362,16 @@
         <v>15.0423611111111</v>
       </c>
       <c r="BY18" s="40" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="BZ18" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="CA18" s="39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="CB18" s="39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="CC18" s="42" t="n">
         <f aca="false">AO18</f>
@@ -7346,7 +7381,7 @@
         <v>15.0423611111111</v>
       </c>
       <c r="CE18" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF18" s="42"/>
       <c r="CG18" s="42"/>
@@ -7374,7 +7409,7 @@
         <v>108</v>
       </c>
       <c r="C19" s="58" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="D19" s="59"/>
       <c r="E19" s="42" t="n">
@@ -7396,69 +7431,72 @@
         <v>113</v>
       </c>
       <c r="K19" s="58" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="L19" s="58" t="s">
-        <v>298</v>
+        <v>301</v>
+      </c>
+      <c r="M19" s="39" t="s">
+        <v>145</v>
       </c>
       <c r="N19" s="58" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O19" s="58" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="P19" s="48" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="Q19" s="43" t="n">
         <v>33314</v>
       </c>
       <c r="R19" s="58" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="S19" s="58" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="T19" s="58"/>
       <c r="U19" s="48"/>
       <c r="V19" s="58" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="W19" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="X19" s="59" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="Y19" s="48" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="Z19" s="59" t="n">
         <v>45669</v>
       </c>
       <c r="AA19" s="59" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="AB19" s="48" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="AC19" s="59" t="n">
         <v>45669</v>
       </c>
       <c r="AD19" s="59" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="AE19" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF19" s="60" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AG19" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AH19" s="58" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="AI19" s="59" t="n">
         <v>45668</v>
@@ -7467,22 +7505,22 @@
         <v>0.732638888888889</v>
       </c>
       <c r="AK19" s="61" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="AL19" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM19" s="62" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="AN19" s="47" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="AO19" s="59" t="n">
         <v>45670</v>
       </c>
       <c r="AP19" s="40" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="AQ19" s="40" t="s">
         <v>123</v>
@@ -7506,7 +7544,7 @@
         <v>3</v>
       </c>
       <c r="AX19" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY19" s="42" t="n">
         <v>45668</v>
@@ -7515,13 +7553,13 @@
         <v>45670</v>
       </c>
       <c r="BA19" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BB19" s="48" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="BC19" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BD19" s="42" t="n">
         <v>45671</v>
@@ -7530,31 +7568,31 @@
         <v>45672</v>
       </c>
       <c r="BF19" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG19" s="40" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="BH19" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI19" s="60"/>
       <c r="BJ19" s="60"/>
       <c r="BK19" s="48"/>
       <c r="BL19" s="48" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="BM19" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN19" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BO19" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP19" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BQ19" s="42" t="n">
         <f aca="false">AL19</f>
@@ -7567,13 +7605,13 @@
         <v>135</v>
       </c>
       <c r="BT19" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BU19" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV19" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BW19" s="42" t="n">
         <f aca="false">AO19</f>
@@ -7583,16 +7621,16 @@
         <v>16.0423611111111</v>
       </c>
       <c r="BY19" s="40" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="BZ19" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="CA19" s="39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="CB19" s="39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="CC19" s="42" t="n">
         <f aca="false">AO19</f>
@@ -7602,7 +7640,7 @@
         <v>16.0423611111111</v>
       </c>
       <c r="CE19" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF19" s="59"/>
       <c r="CG19" s="59"/>
@@ -7627,7 +7665,7 @@
         <v>108</v>
       </c>
       <c r="C20" s="58" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="D20" s="59"/>
       <c r="E20" s="42" t="n">
@@ -7649,19 +7687,22 @@
         <v>113</v>
       </c>
       <c r="K20" s="58" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="L20" s="58" t="s">
-        <v>302</v>
+        <v>305</v>
+      </c>
+      <c r="M20" s="39" t="s">
+        <v>145</v>
       </c>
       <c r="N20" s="58" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="O20" s="58" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="P20" s="48" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="Q20" s="43" t="n">
         <v>33003</v>
@@ -7673,43 +7714,43 @@
       <c r="T20" s="58"/>
       <c r="U20" s="48"/>
       <c r="V20" s="58" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="W20" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="X20" s="59" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="Y20" s="48" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="Z20" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="AA20" s="59" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="AB20" s="48" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="AC20" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="AD20" s="59" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="AE20" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF20" s="60" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AG20" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AH20" s="58" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="AI20" s="59" t="n">
         <v>45668</v>
@@ -7718,22 +7759,22 @@
         <v>0.225694444444444</v>
       </c>
       <c r="AK20" s="61" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="AL20" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM20" s="62" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="AN20" s="47" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="AO20" s="59" t="n">
         <v>45670</v>
       </c>
       <c r="AP20" s="40" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="AQ20" s="40" t="s">
         <v>123</v>
@@ -7757,7 +7798,7 @@
         <v>3</v>
       </c>
       <c r="AX20" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY20" s="42" t="n">
         <v>45668</v>
@@ -7766,13 +7807,13 @@
         <v>45670</v>
       </c>
       <c r="BA20" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BB20" s="48" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BC20" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BD20" s="42" t="n">
         <v>45671</v>
@@ -7781,31 +7822,31 @@
         <v>45672</v>
       </c>
       <c r="BF20" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG20" s="40" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="BH20" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI20" s="60"/>
       <c r="BJ20" s="60"/>
       <c r="BK20" s="48"/>
       <c r="BL20" s="48" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="BM20" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN20" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BO20" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP20" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BQ20" s="42" t="n">
         <f aca="false">AL20</f>
@@ -7818,13 +7859,13 @@
         <v>135</v>
       </c>
       <c r="BT20" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BU20" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV20" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BW20" s="42" t="n">
         <f aca="false">AO20</f>
@@ -7834,16 +7875,16 @@
         <v>17.0423611111111</v>
       </c>
       <c r="BY20" s="40" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="BZ20" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="CA20" s="39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="CB20" s="39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="CC20" s="42" t="n">
         <f aca="false">AO20</f>
@@ -7853,7 +7894,7 @@
         <v>17.0423611111111</v>
       </c>
       <c r="CE20" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF20" s="59"/>
       <c r="CG20" s="59"/>
@@ -7878,7 +7919,7 @@
         <v>108</v>
       </c>
       <c r="C21" s="58" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="D21" s="59"/>
       <c r="E21" s="42" t="n">
@@ -7900,25 +7941,28 @@
         <v>113</v>
       </c>
       <c r="K21" s="58" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="L21" s="58" t="s">
-        <v>314</v>
+        <v>317</v>
+      </c>
+      <c r="M21" s="39" t="s">
+        <v>145</v>
       </c>
       <c r="N21" s="58" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="O21" s="58" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="P21" s="48" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="Q21" s="43" t="n">
         <v>32465</v>
       </c>
       <c r="R21" s="58" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="S21" s="58" t="s">
         <v>120</v>
@@ -7926,43 +7970,43 @@
       <c r="T21" s="58"/>
       <c r="U21" s="48"/>
       <c r="V21" s="58" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="W21" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="X21" s="59" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="Y21" s="48" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="Z21" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="AA21" s="59" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="AB21" s="48" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="AC21" s="59" t="n">
         <v>45668</v>
       </c>
       <c r="AD21" s="59" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="AE21" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AF21" s="60" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AG21" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AH21" s="63" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="AI21" s="55" t="n">
         <v>45668</v>
@@ -7971,22 +8015,22 @@
         <v>0.732638888888889</v>
       </c>
       <c r="AK21" s="61" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="AL21" s="42" t="n">
         <v>45668</v>
       </c>
       <c r="AM21" s="62" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="AN21" s="47" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="AO21" s="59" t="n">
         <v>45670</v>
       </c>
       <c r="AP21" s="40" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="AQ21" s="40" t="s">
         <v>123</v>
@@ -8010,7 +8054,7 @@
         <v>3</v>
       </c>
       <c r="AX21" s="40" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="AY21" s="42" t="n">
         <v>45668</v>
@@ -8019,13 +8063,13 @@
         <v>45670</v>
       </c>
       <c r="BA21" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BB21" s="48" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="BC21" s="40" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="BD21" s="42" t="n">
         <v>45671</v>
@@ -8034,31 +8078,31 @@
         <v>45672</v>
       </c>
       <c r="BF21" s="40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="BG21" s="40" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="BH21" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="BI21" s="60"/>
       <c r="BJ21" s="60"/>
       <c r="BK21" s="48"/>
       <c r="BL21" s="48" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="BM21" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BN21" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BO21" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BP21" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BQ21" s="42" t="n">
         <f aca="false">AL21</f>
@@ -8071,13 +8115,13 @@
         <v>135</v>
       </c>
       <c r="BT21" s="40" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="BU21" s="40" t="s">
         <v>135</v>
       </c>
       <c r="BV21" s="40" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="BW21" s="42" t="n">
         <f aca="false">AO21</f>
@@ -8087,16 +8131,16 @@
         <v>18.0423611111111</v>
       </c>
       <c r="BY21" s="40" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="BZ21" s="42" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="CA21" s="39" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="CB21" s="39" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="CC21" s="42" t="n">
         <f aca="false">AO21</f>
@@ -8106,7 +8150,7 @@
         <v>18.0423611111111</v>
       </c>
       <c r="CE21" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="CF21" s="59"/>
       <c r="CG21" s="59"/>
@@ -29162,10 +29206,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="D1" s="99" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="E1" s="99" t="s">
         <v>4</v>
@@ -29174,13 +29218,13 @@
         <v>5</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H1" s="11" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="15" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="J1" s="15" t="s">
         <v>9</v>
@@ -29195,7 +29239,7 @@
         <v>12</v>
       </c>
       <c r="N1" s="32" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="O1" s="32" t="s">
         <v>14</v>
@@ -29479,7 +29523,7 @@
         <v>115</v>
       </c>
       <c r="M2" s="32" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="N2" s="32" t="s">
         <v>117</v>
@@ -29758,72 +29802,70 @@
         <v>113</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="S3" s="2"/>
       <c r="T3" s="2"/>
       <c r="U3" s="1"/>
       <c r="V3" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="W3" s="5"/>
       <c r="X3" s="1"/>
       <c r="Y3" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="Z3" s="5"/>
       <c r="AA3" s="1"/>
       <c r="AB3" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AD3" s="1"/>
       <c r="AE3" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="AF3" s="5" t="s">
-        <v>147</v>
-      </c>
+        <v>148</v>
+      </c>
+      <c r="AF3" s="5"/>
       <c r="AG3" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="AH3" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="AI3" s="5"/>
+        <v>148</v>
+      </c>
+      <c r="AH3" s="2"/>
+      <c r="AI3" s="1" t="s">
+        <v>148</v>
+      </c>
       <c r="AJ3" s="6"/>
       <c r="AK3" s="1" t="n">
         <v>1</v>
       </c>
       <c r="AL3" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AM3" s="7"/>
       <c r="AN3" s="1"/>
       <c r="AO3" s="5"/>
       <c r="AP3" s="8"/>
       <c r="AQ3" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AR3" s="40"/>
       <c r="AS3" s="40"/>
@@ -29866,7 +29908,7 @@
       <c r="CN3" s="5"/>
       <c r="CO3" s="1"/>
       <c r="CQ3" s="1" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="CR3" s="1"/>
       <c r="CS3" s="1"/>

</xml_diff>